<commit_message>
SQL cleaning phase done (filter under 65, convert hypertension and heart disease to text, drop single gender instance).
</commit_message>
<xml_diff>
--- a/documentation/under65_ai_project_documentations.xlsx
+++ b/documentation/under65_ai_project_documentations.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jarpy\Documents\portfolio_projects\under65_stroke_risk_ai_tool\documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBF0F129-0D75-4229-B8EA-16F4D1A39B44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A74841E1-03A0-4A16-A34D-FA86C1F9A16F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{B009FAC1-510D-4360-8356-4F13549178C2}"/>
+    <workbookView xWindow="-20610" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="2" xr2:uid="{B009FAC1-510D-4360-8356-4F13549178C2}"/>
   </bookViews>
   <sheets>
     <sheet name="Project Overview" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="95">
   <si>
     <t>Under 65 AI Stroke Risk Assessment Tool</t>
   </si>
@@ -397,12 +397,124 @@
     <t>Gender status 'other' was part of the 65 and over population and was already filtered out.
 Decision ot remove the datapoint because it was a single instance that would have potentially created noise in the dataset.</t>
   </si>
+  <si>
+    <t>hypertension column coversion to text</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">hypertension is originally numerical type with 0/1 which may cause a problem when one-hot-coding, therefore the values were replaced with </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>'no_hypertension'</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> and </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>'hypertension'</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>SQL</t>
+  </si>
+  <si>
+    <t>Convert hypertension and heart_disease into text form to preapre for one-hot-coding</t>
+  </si>
+  <si>
+    <t>heart_disease column conversion to text</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">heart_disease is originally numerical type with 0/1 which may cause a problem when one-hot-coding, therefore the values were replaced with </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>'no_heart_disease'</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> and </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>'heart_disease'</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>Create view and download the dataset for python processing.</t>
+  </si>
+  <si>
+    <t>Python</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -438,6 +550,14 @@
       <b/>
       <sz val="14"/>
       <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -493,20 +613,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -525,7 +633,28 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -866,332 +995,332 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:10" ht="18" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="7"/>
+      <c r="G1" s="7"/>
+      <c r="H1" s="7"/>
+      <c r="I1" s="7"/>
+      <c r="J1" s="7"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
-      <c r="H2" s="3"/>
-      <c r="I2" s="3"/>
-      <c r="J2" s="3"/>
+      <c r="B2" s="9"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="9"/>
+      <c r="I2" s="9"/>
+      <c r="J2" s="9"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A3" s="3"/>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
-      <c r="H3" s="3"/>
-      <c r="I3" s="3"/>
-      <c r="J3" s="3"/>
+      <c r="A3" s="9"/>
+      <c r="B3" s="9"/>
+      <c r="C3" s="9"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="9"/>
+      <c r="G3" s="9"/>
+      <c r="H3" s="9"/>
+      <c r="I3" s="9"/>
+      <c r="J3" s="9"/>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A4" s="3"/>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
-      <c r="H4" s="3"/>
-      <c r="I4" s="3"/>
-      <c r="J4" s="3"/>
+      <c r="A4" s="9"/>
+      <c r="B4" s="9"/>
+      <c r="C4" s="9"/>
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="9"/>
+      <c r="G4" s="9"/>
+      <c r="H4" s="9"/>
+      <c r="I4" s="9"/>
+      <c r="J4" s="9"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A5" s="3"/>
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
-      <c r="H5" s="3"/>
-      <c r="I5" s="3"/>
-      <c r="J5" s="3"/>
+      <c r="A5" s="9"/>
+      <c r="B5" s="9"/>
+      <c r="C5" s="9"/>
+      <c r="D5" s="9"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
+      <c r="G5" s="9"/>
+      <c r="H5" s="9"/>
+      <c r="I5" s="9"/>
+      <c r="J5" s="9"/>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A6" s="3"/>
-      <c r="B6" s="3"/>
-      <c r="C6" s="3"/>
-      <c r="D6" s="3"/>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3"/>
-      <c r="G6" s="3"/>
-      <c r="H6" s="3"/>
-      <c r="I6" s="3"/>
-      <c r="J6" s="3"/>
+      <c r="A6" s="9"/>
+      <c r="B6" s="9"/>
+      <c r="C6" s="9"/>
+      <c r="D6" s="9"/>
+      <c r="E6" s="9"/>
+      <c r="F6" s="9"/>
+      <c r="G6" s="9"/>
+      <c r="H6" s="9"/>
+      <c r="I6" s="9"/>
+      <c r="J6" s="9"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A7" s="3"/>
-      <c r="B7" s="3"/>
-      <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3"/>
-      <c r="G7" s="3"/>
-      <c r="H7" s="3"/>
-      <c r="I7" s="3"/>
-      <c r="J7" s="3"/>
+      <c r="A7" s="9"/>
+      <c r="B7" s="9"/>
+      <c r="C7" s="9"/>
+      <c r="D7" s="9"/>
+      <c r="E7" s="9"/>
+      <c r="F7" s="9"/>
+      <c r="G7" s="9"/>
+      <c r="H7" s="9"/>
+      <c r="I7" s="9"/>
+      <c r="J7" s="9"/>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A8" s="3"/>
-      <c r="B8" s="3"/>
-      <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
-      <c r="E8" s="3"/>
-      <c r="F8" s="3"/>
-      <c r="G8" s="3"/>
-      <c r="H8" s="3"/>
-      <c r="I8" s="3"/>
-      <c r="J8" s="3"/>
+      <c r="A8" s="9"/>
+      <c r="B8" s="9"/>
+      <c r="C8" s="9"/>
+      <c r="D8" s="9"/>
+      <c r="E8" s="9"/>
+      <c r="F8" s="9"/>
+      <c r="G8" s="9"/>
+      <c r="H8" s="9"/>
+      <c r="I8" s="9"/>
+      <c r="J8" s="9"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A9" s="3"/>
-      <c r="B9" s="3"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
-      <c r="E9" s="3"/>
-      <c r="F9" s="3"/>
-      <c r="G9" s="3"/>
-      <c r="H9" s="3"/>
-      <c r="I9" s="3"/>
-      <c r="J9" s="3"/>
+      <c r="A9" s="9"/>
+      <c r="B9" s="9"/>
+      <c r="C9" s="9"/>
+      <c r="D9" s="9"/>
+      <c r="E9" s="9"/>
+      <c r="F9" s="9"/>
+      <c r="G9" s="9"/>
+      <c r="H9" s="9"/>
+      <c r="I9" s="9"/>
+      <c r="J9" s="9"/>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A10" s="3"/>
-      <c r="B10" s="3"/>
-      <c r="C10" s="3"/>
-      <c r="D10" s="3"/>
-      <c r="E10" s="3"/>
-      <c r="F10" s="3"/>
-      <c r="G10" s="3"/>
-      <c r="H10" s="3"/>
-      <c r="I10" s="3"/>
-      <c r="J10" s="3"/>
+      <c r="A10" s="9"/>
+      <c r="B10" s="9"/>
+      <c r="C10" s="9"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="9"/>
+      <c r="F10" s="9"/>
+      <c r="G10" s="9"/>
+      <c r="H10" s="9"/>
+      <c r="I10" s="9"/>
+      <c r="J10" s="9"/>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A11" s="3"/>
-      <c r="B11" s="3"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="3"/>
-      <c r="E11" s="3"/>
-      <c r="F11" s="3"/>
-      <c r="G11" s="3"/>
-      <c r="H11" s="3"/>
-      <c r="I11" s="3"/>
-      <c r="J11" s="3"/>
+      <c r="A11" s="9"/>
+      <c r="B11" s="9"/>
+      <c r="C11" s="9"/>
+      <c r="D11" s="9"/>
+      <c r="E11" s="9"/>
+      <c r="F11" s="9"/>
+      <c r="G11" s="9"/>
+      <c r="H11" s="9"/>
+      <c r="I11" s="9"/>
+      <c r="J11" s="9"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="3"/>
-      <c r="B12" s="3"/>
-      <c r="C12" s="3"/>
-      <c r="D12" s="3"/>
-      <c r="E12" s="3"/>
-      <c r="F12" s="3"/>
-      <c r="G12" s="3"/>
-      <c r="H12" s="3"/>
-      <c r="I12" s="3"/>
-      <c r="J12" s="3"/>
+      <c r="A12" s="9"/>
+      <c r="B12" s="9"/>
+      <c r="C12" s="9"/>
+      <c r="D12" s="9"/>
+      <c r="E12" s="9"/>
+      <c r="F12" s="9"/>
+      <c r="G12" s="9"/>
+      <c r="H12" s="9"/>
+      <c r="I12" s="9"/>
+      <c r="J12" s="9"/>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A13" s="3"/>
-      <c r="B13" s="3"/>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
-      <c r="E13" s="3"/>
-      <c r="F13" s="3"/>
-      <c r="G13" s="3"/>
-      <c r="H13" s="3"/>
-      <c r="I13" s="3"/>
-      <c r="J13" s="3"/>
+      <c r="A13" s="9"/>
+      <c r="B13" s="9"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="9"/>
+      <c r="E13" s="9"/>
+      <c r="F13" s="9"/>
+      <c r="G13" s="9"/>
+      <c r="H13" s="9"/>
+      <c r="I13" s="9"/>
+      <c r="J13" s="9"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A14" s="3"/>
-      <c r="B14" s="3"/>
-      <c r="C14" s="3"/>
-      <c r="D14" s="3"/>
-      <c r="E14" s="3"/>
-      <c r="F14" s="3"/>
-      <c r="G14" s="3"/>
-      <c r="H14" s="3"/>
-      <c r="I14" s="3"/>
-      <c r="J14" s="3"/>
+      <c r="A14" s="9"/>
+      <c r="B14" s="9"/>
+      <c r="C14" s="9"/>
+      <c r="D14" s="9"/>
+      <c r="E14" s="9"/>
+      <c r="F14" s="9"/>
+      <c r="G14" s="9"/>
+      <c r="H14" s="9"/>
+      <c r="I14" s="9"/>
+      <c r="J14" s="9"/>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A15" s="3"/>
-      <c r="B15" s="3"/>
-      <c r="C15" s="3"/>
-      <c r="D15" s="3"/>
-      <c r="E15" s="3"/>
-      <c r="F15" s="3"/>
-      <c r="G15" s="3"/>
-      <c r="H15" s="3"/>
-      <c r="I15" s="3"/>
-      <c r="J15" s="3"/>
+      <c r="A15" s="9"/>
+      <c r="B15" s="9"/>
+      <c r="C15" s="9"/>
+      <c r="D15" s="9"/>
+      <c r="E15" s="9"/>
+      <c r="F15" s="9"/>
+      <c r="G15" s="9"/>
+      <c r="H15" s="9"/>
+      <c r="I15" s="9"/>
+      <c r="J15" s="9"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="3"/>
-      <c r="B16" s="3"/>
-      <c r="C16" s="3"/>
-      <c r="D16" s="3"/>
-      <c r="E16" s="3"/>
-      <c r="F16" s="3"/>
-      <c r="G16" s="3"/>
-      <c r="H16" s="3"/>
-      <c r="I16" s="3"/>
-      <c r="J16" s="3"/>
+      <c r="A16" s="9"/>
+      <c r="B16" s="9"/>
+      <c r="C16" s="9"/>
+      <c r="D16" s="9"/>
+      <c r="E16" s="9"/>
+      <c r="F16" s="9"/>
+      <c r="G16" s="9"/>
+      <c r="H16" s="9"/>
+      <c r="I16" s="9"/>
+      <c r="J16" s="9"/>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A17" s="3"/>
-      <c r="B17" s="3"/>
-      <c r="C17" s="3"/>
-      <c r="D17" s="3"/>
-      <c r="E17" s="3"/>
-      <c r="F17" s="3"/>
-      <c r="G17" s="3"/>
-      <c r="H17" s="3"/>
-      <c r="I17" s="3"/>
-      <c r="J17" s="3"/>
+      <c r="A17" s="9"/>
+      <c r="B17" s="9"/>
+      <c r="C17" s="9"/>
+      <c r="D17" s="9"/>
+      <c r="E17" s="9"/>
+      <c r="F17" s="9"/>
+      <c r="G17" s="9"/>
+      <c r="H17" s="9"/>
+      <c r="I17" s="9"/>
+      <c r="J17" s="9"/>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A18" s="3"/>
-      <c r="B18" s="3"/>
-      <c r="C18" s="3"/>
-      <c r="D18" s="3"/>
-      <c r="E18" s="3"/>
-      <c r="F18" s="3"/>
-      <c r="G18" s="3"/>
-      <c r="H18" s="3"/>
-      <c r="I18" s="3"/>
-      <c r="J18" s="3"/>
+      <c r="A18" s="9"/>
+      <c r="B18" s="9"/>
+      <c r="C18" s="9"/>
+      <c r="D18" s="9"/>
+      <c r="E18" s="9"/>
+      <c r="F18" s="9"/>
+      <c r="G18" s="9"/>
+      <c r="H18" s="9"/>
+      <c r="I18" s="9"/>
+      <c r="J18" s="9"/>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A19" s="3"/>
-      <c r="B19" s="3"/>
-      <c r="C19" s="3"/>
-      <c r="D19" s="3"/>
-      <c r="E19" s="3"/>
-      <c r="F19" s="3"/>
-      <c r="G19" s="3"/>
-      <c r="H19" s="3"/>
-      <c r="I19" s="3"/>
-      <c r="J19" s="3"/>
+      <c r="A19" s="9"/>
+      <c r="B19" s="9"/>
+      <c r="C19" s="9"/>
+      <c r="D19" s="9"/>
+      <c r="E19" s="9"/>
+      <c r="F19" s="9"/>
+      <c r="G19" s="9"/>
+      <c r="H19" s="9"/>
+      <c r="I19" s="9"/>
+      <c r="J19" s="9"/>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A20" s="3"/>
-      <c r="B20" s="3"/>
-      <c r="C20" s="3"/>
-      <c r="D20" s="3"/>
-      <c r="E20" s="3"/>
-      <c r="F20" s="3"/>
-      <c r="G20" s="3"/>
-      <c r="H20" s="3"/>
-      <c r="I20" s="3"/>
-      <c r="J20" s="3"/>
+      <c r="A20" s="9"/>
+      <c r="B20" s="9"/>
+      <c r="C20" s="9"/>
+      <c r="D20" s="9"/>
+      <c r="E20" s="9"/>
+      <c r="F20" s="9"/>
+      <c r="G20" s="9"/>
+      <c r="H20" s="9"/>
+      <c r="I20" s="9"/>
+      <c r="J20" s="9"/>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A21" s="3"/>
-      <c r="B21" s="3"/>
-      <c r="C21" s="3"/>
-      <c r="D21" s="3"/>
-      <c r="E21" s="3"/>
-      <c r="F21" s="3"/>
-      <c r="G21" s="3"/>
-      <c r="H21" s="3"/>
-      <c r="I21" s="3"/>
-      <c r="J21" s="3"/>
+      <c r="A21" s="9"/>
+      <c r="B21" s="9"/>
+      <c r="C21" s="9"/>
+      <c r="D21" s="9"/>
+      <c r="E21" s="9"/>
+      <c r="F21" s="9"/>
+      <c r="G21" s="9"/>
+      <c r="H21" s="9"/>
+      <c r="I21" s="9"/>
+      <c r="J21" s="9"/>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A22" s="3"/>
-      <c r="B22" s="3"/>
-      <c r="C22" s="3"/>
-      <c r="D22" s="3"/>
-      <c r="E22" s="3"/>
-      <c r="F22" s="3"/>
-      <c r="G22" s="3"/>
-      <c r="H22" s="3"/>
-      <c r="I22" s="3"/>
-      <c r="J22" s="3"/>
+      <c r="A22" s="9"/>
+      <c r="B22" s="9"/>
+      <c r="C22" s="9"/>
+      <c r="D22" s="9"/>
+      <c r="E22" s="9"/>
+      <c r="F22" s="9"/>
+      <c r="G22" s="9"/>
+      <c r="H22" s="9"/>
+      <c r="I22" s="9"/>
+      <c r="J22" s="9"/>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A23" s="3"/>
-      <c r="B23" s="3"/>
-      <c r="C23" s="3"/>
-      <c r="D23" s="3"/>
-      <c r="E23" s="3"/>
-      <c r="F23" s="3"/>
-      <c r="G23" s="3"/>
-      <c r="H23" s="3"/>
-      <c r="I23" s="3"/>
-      <c r="J23" s="3"/>
+      <c r="A23" s="9"/>
+      <c r="B23" s="9"/>
+      <c r="C23" s="9"/>
+      <c r="D23" s="9"/>
+      <c r="E23" s="9"/>
+      <c r="F23" s="9"/>
+      <c r="G23" s="9"/>
+      <c r="H23" s="9"/>
+      <c r="I23" s="9"/>
+      <c r="J23" s="9"/>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A24" s="3"/>
-      <c r="B24" s="3"/>
-      <c r="C24" s="3"/>
-      <c r="D24" s="3"/>
-      <c r="E24" s="3"/>
-      <c r="F24" s="3"/>
-      <c r="G24" s="3"/>
-      <c r="H24" s="3"/>
-      <c r="I24" s="3"/>
-      <c r="J24" s="3"/>
+      <c r="A24" s="9"/>
+      <c r="B24" s="9"/>
+      <c r="C24" s="9"/>
+      <c r="D24" s="9"/>
+      <c r="E24" s="9"/>
+      <c r="F24" s="9"/>
+      <c r="G24" s="9"/>
+      <c r="H24" s="9"/>
+      <c r="I24" s="9"/>
+      <c r="J24" s="9"/>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A25" s="3"/>
-      <c r="B25" s="3"/>
-      <c r="C25" s="3"/>
-      <c r="D25" s="3"/>
-      <c r="E25" s="3"/>
-      <c r="F25" s="3"/>
-      <c r="G25" s="3"/>
-      <c r="H25" s="3"/>
-      <c r="I25" s="3"/>
-      <c r="J25" s="3"/>
+      <c r="A25" s="9"/>
+      <c r="B25" s="9"/>
+      <c r="C25" s="9"/>
+      <c r="D25" s="9"/>
+      <c r="E25" s="9"/>
+      <c r="F25" s="9"/>
+      <c r="G25" s="9"/>
+      <c r="H25" s="9"/>
+      <c r="I25" s="9"/>
+      <c r="J25" s="9"/>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A26" s="3"/>
-      <c r="B26" s="3"/>
-      <c r="C26" s="3"/>
-      <c r="D26" s="3"/>
-      <c r="E26" s="3"/>
-      <c r="F26" s="3"/>
-      <c r="G26" s="3"/>
-      <c r="H26" s="3"/>
-      <c r="I26" s="3"/>
-      <c r="J26" s="3"/>
+      <c r="A26" s="9"/>
+      <c r="B26" s="9"/>
+      <c r="C26" s="9"/>
+      <c r="D26" s="9"/>
+      <c r="E26" s="9"/>
+      <c r="F26" s="9"/>
+      <c r="G26" s="9"/>
+      <c r="H26" s="9"/>
+      <c r="I26" s="9"/>
+      <c r="J26" s="9"/>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A27" s="3"/>
-      <c r="B27" s="3"/>
-      <c r="C27" s="3"/>
-      <c r="D27" s="3"/>
-      <c r="E27" s="3"/>
-      <c r="F27" s="3"/>
-      <c r="G27" s="3"/>
-      <c r="H27" s="3"/>
-      <c r="I27" s="3"/>
-      <c r="J27" s="3"/>
+      <c r="A27" s="9"/>
+      <c r="B27" s="9"/>
+      <c r="C27" s="9"/>
+      <c r="D27" s="9"/>
+      <c r="E27" s="9"/>
+      <c r="F27" s="9"/>
+      <c r="G27" s="9"/>
+      <c r="H27" s="9"/>
+      <c r="I27" s="9"/>
+      <c r="J27" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1207,281 +1336,281 @@
   <dimension ref="B1:G23"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.88671875" style="5"/>
-    <col min="2" max="2" width="26.5546875" style="5" customWidth="1"/>
-    <col min="3" max="3" width="17.6640625" style="5" customWidth="1"/>
-    <col min="4" max="4" width="35.77734375" style="5" customWidth="1"/>
-    <col min="5" max="5" width="35.44140625" style="5" customWidth="1"/>
-    <col min="6" max="6" width="26.6640625" style="5" customWidth="1"/>
-    <col min="7" max="7" width="53" style="5" customWidth="1"/>
-    <col min="8" max="16384" width="8.88671875" style="5"/>
+    <col min="1" max="1" width="8.88671875" style="1"/>
+    <col min="2" max="2" width="26.5546875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="17.6640625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="35.77734375" style="1" customWidth="1"/>
+    <col min="5" max="5" width="35.44140625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="26.6640625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="53" style="1" customWidth="1"/>
+    <col min="8" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:7" ht="21" x14ac:dyDescent="0.3">
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-    </row>
-    <row r="2" spans="2:7" s="7" customFormat="1" ht="18" x14ac:dyDescent="0.3">
-      <c r="B2" s="9" t="s">
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="10"/>
+      <c r="F1" s="10"/>
+      <c r="G1" s="10"/>
+    </row>
+    <row r="2" spans="2:7" s="3" customFormat="1" ht="18" x14ac:dyDescent="0.3">
+      <c r="B2" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="9" t="s">
+      <c r="C2" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="D2" s="9" t="s">
+      <c r="D2" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="E2" s="9" t="s">
+      <c r="E2" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="F2" s="9" t="s">
+      <c r="F2" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="G2" s="9" t="s">
+      <c r="G2" s="5" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="3" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="E3" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="F3" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="G3" s="6"/>
+      <c r="G3" s="2"/>
     </row>
     <row r="4" spans="2:7" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="D4" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="E4" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="F4" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="G4" s="10" t="s">
+      <c r="G4" s="6" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="5" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D5" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="E5" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F5" s="6" t="s">
+      <c r="F5" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="G5" s="6" t="s">
+      <c r="G5" s="2" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="6" spans="2:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="D6" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="E6" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="F6" s="6" t="s">
+      <c r="F6" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="G6" s="6" t="s">
+      <c r="G6" s="2" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="7" spans="2:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="D7" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="E7" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="F7" s="6" t="s">
+      <c r="F7" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="G7" s="6" t="s">
+      <c r="G7" s="2" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="8" spans="2:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="C8" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="D8" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="E8" s="6" t="s">
+      <c r="E8" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="F8" s="6" t="s">
+      <c r="F8" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="G8" s="6" t="s">
+      <c r="G8" s="2" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="9" spans="2:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="C9" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="D9" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="E9" s="6" t="s">
+      <c r="E9" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="F9" s="6" t="s">
+      <c r="F9" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="G9" s="6" t="s">
+      <c r="G9" s="2" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="10" spans="2:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B10" s="6" t="s">
+      <c r="B10" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="C10" s="6" t="s">
+      <c r="C10" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="D10" s="6" t="s">
+      <c r="D10" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="E10" s="6" t="s">
+      <c r="E10" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="F10" s="6" t="s">
+      <c r="F10" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="G10" s="6" t="s">
+      <c r="G10" s="2" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="11" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="C11" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="D11" s="6" t="s">
+      <c r="D11" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="E11" s="6" t="s">
+      <c r="E11" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F11" s="6" t="s">
+      <c r="F11" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="G11" s="6" t="s">
+      <c r="G11" s="2" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="12" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B12" s="6" t="s">
+      <c r="B12" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="C12" s="6" t="s">
+      <c r="C12" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="D12" s="6" t="s">
+      <c r="D12" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="E12" s="6" t="s">
+      <c r="E12" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F12" s="6" t="s">
+      <c r="F12" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="G12" s="6" t="s">
+      <c r="G12" s="2" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="13" spans="2:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B13" s="6" t="s">
+      <c r="B13" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="C13" s="6" t="s">
+      <c r="C13" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="D13" s="6" t="s">
+      <c r="D13" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="E13" s="6" t="s">
+      <c r="E13" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="F13" s="6" t="s">
+      <c r="F13" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="G13" s="6" t="s">
+      <c r="G13" s="2" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="14" spans="2:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B14" s="6" t="s">
+      <c r="B14" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="C14" s="6" t="s">
+      <c r="C14" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="D14" s="6" t="s">
+      <c r="D14" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="E14" s="6" t="s">
+      <c r="E14" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="F14" s="6" t="s">
+      <c r="F14" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="G14" s="6" t="s">
+      <c r="G14" s="2" t="s">
         <v>55</v>
       </c>
     </row>
@@ -1496,150 +1625,150 @@
       <c r="G15" s="11"/>
     </row>
     <row r="16" spans="2:7" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="9" t="s">
+      <c r="B16" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C16" s="9" t="s">
+      <c r="C16" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="D16" s="9" t="s">
+      <c r="D16" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="E16" s="9" t="s">
+      <c r="E16" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="F16" s="9" t="s">
+      <c r="F16" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="G16" s="9" t="s">
+      <c r="G16" s="5" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="17" spans="2:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B17" s="6" t="s">
+      <c r="B17" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="C17" s="6" t="s">
+      <c r="C17" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="D17" s="6" t="s">
+      <c r="D17" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="E17" s="6" t="s">
+      <c r="E17" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="F17" s="6" t="s">
+      <c r="F17" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="G17" s="6"/>
+      <c r="G17" s="2"/>
     </row>
     <row r="18" spans="2:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B18" s="6" t="s">
+      <c r="B18" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="C18" s="6" t="s">
+      <c r="C18" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="D18" s="6" t="s">
+      <c r="D18" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="E18" s="6" t="s">
+      <c r="E18" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="F18" s="6" t="s">
+      <c r="F18" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="G18" s="6"/>
+      <c r="G18" s="2"/>
     </row>
     <row r="19" spans="2:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B19" s="6" t="s">
+      <c r="B19" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="C19" s="6" t="s">
+      <c r="C19" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="D19" s="6" t="s">
+      <c r="D19" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="E19" s="6" t="s">
+      <c r="E19" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="F19" s="6" t="s">
+      <c r="F19" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="G19" s="6"/>
+      <c r="G19" s="2"/>
     </row>
     <row r="20" spans="2:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B20" s="6" t="s">
+      <c r="B20" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="C20" s="6" t="s">
+      <c r="C20" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="D20" s="6" t="s">
+      <c r="D20" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="E20" s="6" t="s">
+      <c r="E20" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="F20" s="6" t="s">
+      <c r="F20" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="G20" s="6"/>
+      <c r="G20" s="2"/>
     </row>
     <row r="21" spans="2:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B21" s="6" t="s">
+      <c r="B21" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="C21" s="6" t="s">
+      <c r="C21" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="D21" s="6" t="s">
+      <c r="D21" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="E21" s="6" t="s">
+      <c r="E21" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="F21" s="6" t="s">
+      <c r="F21" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="G21" s="6"/>
+      <c r="G21" s="2"/>
     </row>
     <row r="22" spans="2:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B22" s="6" t="s">
+      <c r="B22" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="C22" s="6" t="s">
+      <c r="C22" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="D22" s="6" t="s">
+      <c r="D22" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="E22" s="6" t="s">
+      <c r="E22" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="F22" s="6" t="s">
+      <c r="F22" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="G22" s="6"/>
+      <c r="G22" s="2"/>
     </row>
     <row r="23" spans="2:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B23" s="6" t="s">
+      <c r="B23" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="C23" s="6" t="s">
+      <c r="C23" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="D23" s="6" t="s">
+      <c r="D23" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="E23" s="6" t="s">
+      <c r="E23" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="F23" s="6" t="s">
+      <c r="F23" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="G23" s="6"/>
+      <c r="G23" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1653,76 +1782,160 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C959EE4-029A-4AE9-A45E-FBFB9C63ADEB}">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.88671875" style="7"/>
-    <col min="2" max="2" width="17.6640625" style="8" customWidth="1"/>
-    <col min="3" max="3" width="26.5546875" style="5" customWidth="1"/>
-    <col min="4" max="4" width="62.6640625" style="5" customWidth="1"/>
-    <col min="5" max="5" width="17.88671875" style="7" customWidth="1"/>
-    <col min="6" max="6" width="44.21875" style="5" customWidth="1"/>
-    <col min="7" max="16384" width="8.88671875" style="5"/>
+    <col min="1" max="1" width="8.88671875" style="3"/>
+    <col min="2" max="2" width="17.6640625" style="4" customWidth="1"/>
+    <col min="3" max="3" width="26.5546875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="62.6640625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="17.88671875" style="3" customWidth="1"/>
+    <col min="6" max="6" width="44.21875" style="1" customWidth="1"/>
+    <col min="7" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="7" t="s">
+    <row r="1" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A1" s="13" t="s">
+        <v>89</v>
+      </c>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+    </row>
+    <row r="2" spans="1:6" s="3" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="14" t="s">
         <v>77</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B2" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C2" s="14" t="s">
         <v>5</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="D2" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="E2" s="14" t="s">
         <v>79</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="F2" s="14" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A2" s="7">
+    <row r="3" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A3" s="3">
         <v>1</v>
       </c>
-      <c r="B2" s="8">
+      <c r="B3" s="4">
         <v>45846</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C3" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="D3" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="E2" s="7" t="s">
+      <c r="E3" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="F3" s="1" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A3" s="7">
+    <row r="4" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A4" s="3">
         <v>2</v>
       </c>
-      <c r="B3" s="8">
+      <c r="B4" s="4">
         <v>45846</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C4" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D4" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="E4" s="3" t="s">
         <v>82</v>
       </c>
+      <c r="F4" s="1" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A5" s="3">
+        <v>3</v>
+      </c>
+      <c r="B5" s="4">
+        <v>45846</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A6" s="3">
+        <v>4</v>
+      </c>
+      <c r="B6" s="4">
+        <v>45846</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" s="12" t="s">
+        <v>94</v>
+      </c>
+      <c r="B7" s="12"/>
+      <c r="C7" s="12"/>
+      <c r="D7" s="12"/>
+      <c r="E7" s="12"/>
+      <c r="F7" s="12"/>
+    </row>
+    <row r="8" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A8" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="B8" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="C8" s="14" t="s">
+        <v>5</v>
+      </c>
+      <c r="D8" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="E8" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="F8" s="14" t="s">
+        <v>80</v>
+      </c>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A7:F7"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Python project and venv created. Utils.data_io created to facilitate data saving and loading. Initial data cleaning process completed.
</commit_message>
<xml_diff>
--- a/documentation/under65_ai_project_documentations.xlsx
+++ b/documentation/under65_ai_project_documentations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jarpy\Documents\portfolio_projects\under65_stroke_risk_ai_tool\documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A74841E1-03A0-4A16-A34D-FA86C1F9A16F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD8A912B-843A-43C2-BBBB-D00BB4A253C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-20610" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="2" xr2:uid="{B009FAC1-510D-4360-8356-4F13549178C2}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="102">
   <si>
     <t>Under 65 AI Stroke Risk Assessment Tool</t>
   </si>
@@ -508,6 +508,30 @@
   </si>
   <si>
     <t>Python</t>
+  </si>
+  <si>
+    <t>Comments &amp; Insights</t>
+  </si>
+  <si>
+    <t>Dataset Info</t>
+  </si>
+  <si>
+    <t>1. 4083 rows for every feature except BMI that contains 127 null values.
+2. avg_glucose_level summary seems to suggest right skew with max value of 267 and Q3 value of 111.
+3. BMI shows extreme right skew with Q3 of 33 and max of 97
+4. From previous project iteration, outliers are present but deemed medically possible; thus, no outliers removed or excluded.</t>
+  </si>
+  <si>
+    <t>Standardize text column</t>
+  </si>
+  <si>
+    <t>Standardized 7 text columns by lowercase, trim, and replacing spaces with underscore.</t>
+  </si>
+  <si>
+    <t>Remove duplicates</t>
+  </si>
+  <si>
+    <t>No duplicates found (excluding id).</t>
   </si>
 </sst>
 </file>
@@ -613,7 +637,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -633,6 +657,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -648,14 +675,20 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -995,332 +1028,332 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:10" ht="18" x14ac:dyDescent="0.35">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
-      <c r="F1" s="7"/>
-      <c r="G1" s="7"/>
-      <c r="H1" s="7"/>
-      <c r="I1" s="7"/>
-      <c r="J1" s="7"/>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="8"/>
+      <c r="H1" s="8"/>
+      <c r="I1" s="8"/>
+      <c r="J1" s="8"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A2" s="8" t="s">
+      <c r="A2" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="9"/>
-      <c r="C2" s="9"/>
-      <c r="D2" s="9"/>
-      <c r="E2" s="9"/>
-      <c r="F2" s="9"/>
-      <c r="G2" s="9"/>
-      <c r="H2" s="9"/>
-      <c r="I2" s="9"/>
-      <c r="J2" s="9"/>
+      <c r="B2" s="10"/>
+      <c r="C2" s="10"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="10"/>
+      <c r="F2" s="10"/>
+      <c r="G2" s="10"/>
+      <c r="H2" s="10"/>
+      <c r="I2" s="10"/>
+      <c r="J2" s="10"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A3" s="9"/>
-      <c r="B3" s="9"/>
-      <c r="C3" s="9"/>
-      <c r="D3" s="9"/>
-      <c r="E3" s="9"/>
-      <c r="F3" s="9"/>
-      <c r="G3" s="9"/>
-      <c r="H3" s="9"/>
-      <c r="I3" s="9"/>
-      <c r="J3" s="9"/>
+      <c r="A3" s="10"/>
+      <c r="B3" s="10"/>
+      <c r="C3" s="10"/>
+      <c r="D3" s="10"/>
+      <c r="E3" s="10"/>
+      <c r="F3" s="10"/>
+      <c r="G3" s="10"/>
+      <c r="H3" s="10"/>
+      <c r="I3" s="10"/>
+      <c r="J3" s="10"/>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A4" s="9"/>
-      <c r="B4" s="9"/>
-      <c r="C4" s="9"/>
-      <c r="D4" s="9"/>
-      <c r="E4" s="9"/>
-      <c r="F4" s="9"/>
-      <c r="G4" s="9"/>
-      <c r="H4" s="9"/>
-      <c r="I4" s="9"/>
-      <c r="J4" s="9"/>
+      <c r="A4" s="10"/>
+      <c r="B4" s="10"/>
+      <c r="C4" s="10"/>
+      <c r="D4" s="10"/>
+      <c r="E4" s="10"/>
+      <c r="F4" s="10"/>
+      <c r="G4" s="10"/>
+      <c r="H4" s="10"/>
+      <c r="I4" s="10"/>
+      <c r="J4" s="10"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A5" s="9"/>
-      <c r="B5" s="9"/>
-      <c r="C5" s="9"/>
-      <c r="D5" s="9"/>
-      <c r="E5" s="9"/>
-      <c r="F5" s="9"/>
-      <c r="G5" s="9"/>
-      <c r="H5" s="9"/>
-      <c r="I5" s="9"/>
-      <c r="J5" s="9"/>
+      <c r="A5" s="10"/>
+      <c r="B5" s="10"/>
+      <c r="C5" s="10"/>
+      <c r="D5" s="10"/>
+      <c r="E5" s="10"/>
+      <c r="F5" s="10"/>
+      <c r="G5" s="10"/>
+      <c r="H5" s="10"/>
+      <c r="I5" s="10"/>
+      <c r="J5" s="10"/>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A6" s="9"/>
-      <c r="B6" s="9"/>
-      <c r="C6" s="9"/>
-      <c r="D6" s="9"/>
-      <c r="E6" s="9"/>
-      <c r="F6" s="9"/>
-      <c r="G6" s="9"/>
-      <c r="H6" s="9"/>
-      <c r="I6" s="9"/>
-      <c r="J6" s="9"/>
+      <c r="A6" s="10"/>
+      <c r="B6" s="10"/>
+      <c r="C6" s="10"/>
+      <c r="D6" s="10"/>
+      <c r="E6" s="10"/>
+      <c r="F6" s="10"/>
+      <c r="G6" s="10"/>
+      <c r="H6" s="10"/>
+      <c r="I6" s="10"/>
+      <c r="J6" s="10"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A7" s="9"/>
-      <c r="B7" s="9"/>
-      <c r="C7" s="9"/>
-      <c r="D7" s="9"/>
-      <c r="E7" s="9"/>
-      <c r="F7" s="9"/>
-      <c r="G7" s="9"/>
-      <c r="H7" s="9"/>
-      <c r="I7" s="9"/>
-      <c r="J7" s="9"/>
+      <c r="A7" s="10"/>
+      <c r="B7" s="10"/>
+      <c r="C7" s="10"/>
+      <c r="D7" s="10"/>
+      <c r="E7" s="10"/>
+      <c r="F7" s="10"/>
+      <c r="G7" s="10"/>
+      <c r="H7" s="10"/>
+      <c r="I7" s="10"/>
+      <c r="J7" s="10"/>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A8" s="9"/>
-      <c r="B8" s="9"/>
-      <c r="C8" s="9"/>
-      <c r="D8" s="9"/>
-      <c r="E8" s="9"/>
-      <c r="F8" s="9"/>
-      <c r="G8" s="9"/>
-      <c r="H8" s="9"/>
-      <c r="I8" s="9"/>
-      <c r="J8" s="9"/>
+      <c r="A8" s="10"/>
+      <c r="B8" s="10"/>
+      <c r="C8" s="10"/>
+      <c r="D8" s="10"/>
+      <c r="E8" s="10"/>
+      <c r="F8" s="10"/>
+      <c r="G8" s="10"/>
+      <c r="H8" s="10"/>
+      <c r="I8" s="10"/>
+      <c r="J8" s="10"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A9" s="9"/>
-      <c r="B9" s="9"/>
-      <c r="C9" s="9"/>
-      <c r="D9" s="9"/>
-      <c r="E9" s="9"/>
-      <c r="F9" s="9"/>
-      <c r="G9" s="9"/>
-      <c r="H9" s="9"/>
-      <c r="I9" s="9"/>
-      <c r="J9" s="9"/>
+      <c r="A9" s="10"/>
+      <c r="B9" s="10"/>
+      <c r="C9" s="10"/>
+      <c r="D9" s="10"/>
+      <c r="E9" s="10"/>
+      <c r="F9" s="10"/>
+      <c r="G9" s="10"/>
+      <c r="H9" s="10"/>
+      <c r="I9" s="10"/>
+      <c r="J9" s="10"/>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A10" s="9"/>
-      <c r="B10" s="9"/>
-      <c r="C10" s="9"/>
-      <c r="D10" s="9"/>
-      <c r="E10" s="9"/>
-      <c r="F10" s="9"/>
-      <c r="G10" s="9"/>
-      <c r="H10" s="9"/>
-      <c r="I10" s="9"/>
-      <c r="J10" s="9"/>
+      <c r="A10" s="10"/>
+      <c r="B10" s="10"/>
+      <c r="C10" s="10"/>
+      <c r="D10" s="10"/>
+      <c r="E10" s="10"/>
+      <c r="F10" s="10"/>
+      <c r="G10" s="10"/>
+      <c r="H10" s="10"/>
+      <c r="I10" s="10"/>
+      <c r="J10" s="10"/>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A11" s="9"/>
-      <c r="B11" s="9"/>
-      <c r="C11" s="9"/>
-      <c r="D11" s="9"/>
-      <c r="E11" s="9"/>
-      <c r="F11" s="9"/>
-      <c r="G11" s="9"/>
-      <c r="H11" s="9"/>
-      <c r="I11" s="9"/>
-      <c r="J11" s="9"/>
+      <c r="A11" s="10"/>
+      <c r="B11" s="10"/>
+      <c r="C11" s="10"/>
+      <c r="D11" s="10"/>
+      <c r="E11" s="10"/>
+      <c r="F11" s="10"/>
+      <c r="G11" s="10"/>
+      <c r="H11" s="10"/>
+      <c r="I11" s="10"/>
+      <c r="J11" s="10"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="9"/>
-      <c r="B12" s="9"/>
-      <c r="C12" s="9"/>
-      <c r="D12" s="9"/>
-      <c r="E12" s="9"/>
-      <c r="F12" s="9"/>
-      <c r="G12" s="9"/>
-      <c r="H12" s="9"/>
-      <c r="I12" s="9"/>
-      <c r="J12" s="9"/>
+      <c r="A12" s="10"/>
+      <c r="B12" s="10"/>
+      <c r="C12" s="10"/>
+      <c r="D12" s="10"/>
+      <c r="E12" s="10"/>
+      <c r="F12" s="10"/>
+      <c r="G12" s="10"/>
+      <c r="H12" s="10"/>
+      <c r="I12" s="10"/>
+      <c r="J12" s="10"/>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A13" s="9"/>
-      <c r="B13" s="9"/>
-      <c r="C13" s="9"/>
-      <c r="D13" s="9"/>
-      <c r="E13" s="9"/>
-      <c r="F13" s="9"/>
-      <c r="G13" s="9"/>
-      <c r="H13" s="9"/>
-      <c r="I13" s="9"/>
-      <c r="J13" s="9"/>
+      <c r="A13" s="10"/>
+      <c r="B13" s="10"/>
+      <c r="C13" s="10"/>
+      <c r="D13" s="10"/>
+      <c r="E13" s="10"/>
+      <c r="F13" s="10"/>
+      <c r="G13" s="10"/>
+      <c r="H13" s="10"/>
+      <c r="I13" s="10"/>
+      <c r="J13" s="10"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A14" s="9"/>
-      <c r="B14" s="9"/>
-      <c r="C14" s="9"/>
-      <c r="D14" s="9"/>
-      <c r="E14" s="9"/>
-      <c r="F14" s="9"/>
-      <c r="G14" s="9"/>
-      <c r="H14" s="9"/>
-      <c r="I14" s="9"/>
-      <c r="J14" s="9"/>
+      <c r="A14" s="10"/>
+      <c r="B14" s="10"/>
+      <c r="C14" s="10"/>
+      <c r="D14" s="10"/>
+      <c r="E14" s="10"/>
+      <c r="F14" s="10"/>
+      <c r="G14" s="10"/>
+      <c r="H14" s="10"/>
+      <c r="I14" s="10"/>
+      <c r="J14" s="10"/>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A15" s="9"/>
-      <c r="B15" s="9"/>
-      <c r="C15" s="9"/>
-      <c r="D15" s="9"/>
-      <c r="E15" s="9"/>
-      <c r="F15" s="9"/>
-      <c r="G15" s="9"/>
-      <c r="H15" s="9"/>
-      <c r="I15" s="9"/>
-      <c r="J15" s="9"/>
+      <c r="A15" s="10"/>
+      <c r="B15" s="10"/>
+      <c r="C15" s="10"/>
+      <c r="D15" s="10"/>
+      <c r="E15" s="10"/>
+      <c r="F15" s="10"/>
+      <c r="G15" s="10"/>
+      <c r="H15" s="10"/>
+      <c r="I15" s="10"/>
+      <c r="J15" s="10"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="9"/>
-      <c r="B16" s="9"/>
-      <c r="C16" s="9"/>
-      <c r="D16" s="9"/>
-      <c r="E16" s="9"/>
-      <c r="F16" s="9"/>
-      <c r="G16" s="9"/>
-      <c r="H16" s="9"/>
-      <c r="I16" s="9"/>
-      <c r="J16" s="9"/>
+      <c r="A16" s="10"/>
+      <c r="B16" s="10"/>
+      <c r="C16" s="10"/>
+      <c r="D16" s="10"/>
+      <c r="E16" s="10"/>
+      <c r="F16" s="10"/>
+      <c r="G16" s="10"/>
+      <c r="H16" s="10"/>
+      <c r="I16" s="10"/>
+      <c r="J16" s="10"/>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A17" s="9"/>
-      <c r="B17" s="9"/>
-      <c r="C17" s="9"/>
-      <c r="D17" s="9"/>
-      <c r="E17" s="9"/>
-      <c r="F17" s="9"/>
-      <c r="G17" s="9"/>
-      <c r="H17" s="9"/>
-      <c r="I17" s="9"/>
-      <c r="J17" s="9"/>
+      <c r="A17" s="10"/>
+      <c r="B17" s="10"/>
+      <c r="C17" s="10"/>
+      <c r="D17" s="10"/>
+      <c r="E17" s="10"/>
+      <c r="F17" s="10"/>
+      <c r="G17" s="10"/>
+      <c r="H17" s="10"/>
+      <c r="I17" s="10"/>
+      <c r="J17" s="10"/>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A18" s="9"/>
-      <c r="B18" s="9"/>
-      <c r="C18" s="9"/>
-      <c r="D18" s="9"/>
-      <c r="E18" s="9"/>
-      <c r="F18" s="9"/>
-      <c r="G18" s="9"/>
-      <c r="H18" s="9"/>
-      <c r="I18" s="9"/>
-      <c r="J18" s="9"/>
+      <c r="A18" s="10"/>
+      <c r="B18" s="10"/>
+      <c r="C18" s="10"/>
+      <c r="D18" s="10"/>
+      <c r="E18" s="10"/>
+      <c r="F18" s="10"/>
+      <c r="G18" s="10"/>
+      <c r="H18" s="10"/>
+      <c r="I18" s="10"/>
+      <c r="J18" s="10"/>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A19" s="9"/>
-      <c r="B19" s="9"/>
-      <c r="C19" s="9"/>
-      <c r="D19" s="9"/>
-      <c r="E19" s="9"/>
-      <c r="F19" s="9"/>
-      <c r="G19" s="9"/>
-      <c r="H19" s="9"/>
-      <c r="I19" s="9"/>
-      <c r="J19" s="9"/>
+      <c r="A19" s="10"/>
+      <c r="B19" s="10"/>
+      <c r="C19" s="10"/>
+      <c r="D19" s="10"/>
+      <c r="E19" s="10"/>
+      <c r="F19" s="10"/>
+      <c r="G19" s="10"/>
+      <c r="H19" s="10"/>
+      <c r="I19" s="10"/>
+      <c r="J19" s="10"/>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A20" s="9"/>
-      <c r="B20" s="9"/>
-      <c r="C20" s="9"/>
-      <c r="D20" s="9"/>
-      <c r="E20" s="9"/>
-      <c r="F20" s="9"/>
-      <c r="G20" s="9"/>
-      <c r="H20" s="9"/>
-      <c r="I20" s="9"/>
-      <c r="J20" s="9"/>
+      <c r="A20" s="10"/>
+      <c r="B20" s="10"/>
+      <c r="C20" s="10"/>
+      <c r="D20" s="10"/>
+      <c r="E20" s="10"/>
+      <c r="F20" s="10"/>
+      <c r="G20" s="10"/>
+      <c r="H20" s="10"/>
+      <c r="I20" s="10"/>
+      <c r="J20" s="10"/>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A21" s="9"/>
-      <c r="B21" s="9"/>
-      <c r="C21" s="9"/>
-      <c r="D21" s="9"/>
-      <c r="E21" s="9"/>
-      <c r="F21" s="9"/>
-      <c r="G21" s="9"/>
-      <c r="H21" s="9"/>
-      <c r="I21" s="9"/>
-      <c r="J21" s="9"/>
+      <c r="A21" s="10"/>
+      <c r="B21" s="10"/>
+      <c r="C21" s="10"/>
+      <c r="D21" s="10"/>
+      <c r="E21" s="10"/>
+      <c r="F21" s="10"/>
+      <c r="G21" s="10"/>
+      <c r="H21" s="10"/>
+      <c r="I21" s="10"/>
+      <c r="J21" s="10"/>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A22" s="9"/>
-      <c r="B22" s="9"/>
-      <c r="C22" s="9"/>
-      <c r="D22" s="9"/>
-      <c r="E22" s="9"/>
-      <c r="F22" s="9"/>
-      <c r="G22" s="9"/>
-      <c r="H22" s="9"/>
-      <c r="I22" s="9"/>
-      <c r="J22" s="9"/>
+      <c r="A22" s="10"/>
+      <c r="B22" s="10"/>
+      <c r="C22" s="10"/>
+      <c r="D22" s="10"/>
+      <c r="E22" s="10"/>
+      <c r="F22" s="10"/>
+      <c r="G22" s="10"/>
+      <c r="H22" s="10"/>
+      <c r="I22" s="10"/>
+      <c r="J22" s="10"/>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A23" s="9"/>
-      <c r="B23" s="9"/>
-      <c r="C23" s="9"/>
-      <c r="D23" s="9"/>
-      <c r="E23" s="9"/>
-      <c r="F23" s="9"/>
-      <c r="G23" s="9"/>
-      <c r="H23" s="9"/>
-      <c r="I23" s="9"/>
-      <c r="J23" s="9"/>
+      <c r="A23" s="10"/>
+      <c r="B23" s="10"/>
+      <c r="C23" s="10"/>
+      <c r="D23" s="10"/>
+      <c r="E23" s="10"/>
+      <c r="F23" s="10"/>
+      <c r="G23" s="10"/>
+      <c r="H23" s="10"/>
+      <c r="I23" s="10"/>
+      <c r="J23" s="10"/>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A24" s="9"/>
-      <c r="B24" s="9"/>
-      <c r="C24" s="9"/>
-      <c r="D24" s="9"/>
-      <c r="E24" s="9"/>
-      <c r="F24" s="9"/>
-      <c r="G24" s="9"/>
-      <c r="H24" s="9"/>
-      <c r="I24" s="9"/>
-      <c r="J24" s="9"/>
+      <c r="A24" s="10"/>
+      <c r="B24" s="10"/>
+      <c r="C24" s="10"/>
+      <c r="D24" s="10"/>
+      <c r="E24" s="10"/>
+      <c r="F24" s="10"/>
+      <c r="G24" s="10"/>
+      <c r="H24" s="10"/>
+      <c r="I24" s="10"/>
+      <c r="J24" s="10"/>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A25" s="9"/>
-      <c r="B25" s="9"/>
-      <c r="C25" s="9"/>
-      <c r="D25" s="9"/>
-      <c r="E25" s="9"/>
-      <c r="F25" s="9"/>
-      <c r="G25" s="9"/>
-      <c r="H25" s="9"/>
-      <c r="I25" s="9"/>
-      <c r="J25" s="9"/>
+      <c r="A25" s="10"/>
+      <c r="B25" s="10"/>
+      <c r="C25" s="10"/>
+      <c r="D25" s="10"/>
+      <c r="E25" s="10"/>
+      <c r="F25" s="10"/>
+      <c r="G25" s="10"/>
+      <c r="H25" s="10"/>
+      <c r="I25" s="10"/>
+      <c r="J25" s="10"/>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A26" s="9"/>
-      <c r="B26" s="9"/>
-      <c r="C26" s="9"/>
-      <c r="D26" s="9"/>
-      <c r="E26" s="9"/>
-      <c r="F26" s="9"/>
-      <c r="G26" s="9"/>
-      <c r="H26" s="9"/>
-      <c r="I26" s="9"/>
-      <c r="J26" s="9"/>
+      <c r="A26" s="10"/>
+      <c r="B26" s="10"/>
+      <c r="C26" s="10"/>
+      <c r="D26" s="10"/>
+      <c r="E26" s="10"/>
+      <c r="F26" s="10"/>
+      <c r="G26" s="10"/>
+      <c r="H26" s="10"/>
+      <c r="I26" s="10"/>
+      <c r="J26" s="10"/>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A27" s="9"/>
-      <c r="B27" s="9"/>
-      <c r="C27" s="9"/>
-      <c r="D27" s="9"/>
-      <c r="E27" s="9"/>
-      <c r="F27" s="9"/>
-      <c r="G27" s="9"/>
-      <c r="H27" s="9"/>
-      <c r="I27" s="9"/>
-      <c r="J27" s="9"/>
+      <c r="A27" s="10"/>
+      <c r="B27" s="10"/>
+      <c r="C27" s="10"/>
+      <c r="D27" s="10"/>
+      <c r="E27" s="10"/>
+      <c r="F27" s="10"/>
+      <c r="G27" s="10"/>
+      <c r="H27" s="10"/>
+      <c r="I27" s="10"/>
+      <c r="J27" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1347,14 +1380,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:7" ht="21" x14ac:dyDescent="0.3">
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10"/>
-      <c r="F1" s="10"/>
-      <c r="G1" s="10"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
+      <c r="F1" s="11"/>
+      <c r="G1" s="11"/>
     </row>
     <row r="2" spans="2:7" s="3" customFormat="1" ht="18" x14ac:dyDescent="0.3">
       <c r="B2" s="5" t="s">
@@ -1615,14 +1648,14 @@
       </c>
     </row>
     <row r="15" spans="2:7" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="11" t="s">
+      <c r="B15" s="12" t="s">
         <v>56</v>
       </c>
-      <c r="C15" s="11"/>
-      <c r="D15" s="11"/>
-      <c r="E15" s="11"/>
-      <c r="F15" s="11"/>
-      <c r="G15" s="11"/>
+      <c r="C15" s="12"/>
+      <c r="D15" s="12"/>
+      <c r="E15" s="12"/>
+      <c r="F15" s="12"/>
+      <c r="G15" s="12"/>
     </row>
     <row r="16" spans="2:7" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="5" t="s">
@@ -1782,7 +1815,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C959EE4-029A-4AE9-A45E-FBFB9C63ADEB}">
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.88671875" style="3"/>
@@ -1805,22 +1838,22 @@
       <c r="F1" s="13"/>
     </row>
     <row r="2" spans="1:6" s="3" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="B2" s="14" t="s">
+      <c r="B2" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="C2" s="14" t="s">
+      <c r="C2" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="14" t="s">
+      <c r="D2" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="14" t="s">
+      <c r="E2" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="F2" s="14" t="s">
+      <c r="F2" s="7" t="s">
         <v>80</v>
       </c>
     </row>
@@ -1902,33 +1935,67 @@
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" s="12" t="s">
+      <c r="A7" s="14" t="s">
         <v>94</v>
       </c>
-      <c r="B7" s="12"/>
-      <c r="C7" s="12"/>
-      <c r="D7" s="12"/>
-      <c r="E7" s="12"/>
-      <c r="F7" s="12"/>
+      <c r="B7" s="14"/>
+      <c r="C7" s="14"/>
+      <c r="D7" s="14"/>
+      <c r="E7" s="14"/>
+      <c r="F7" s="14"/>
     </row>
     <row r="8" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A8" s="14" t="s">
+      <c r="A8" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="B8" s="14" t="s">
+      <c r="B8" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="C8" s="14" t="s">
+      <c r="C8" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="D8" s="14" t="s">
+      <c r="D8" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="E8" s="14" t="s">
+      <c r="E8" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="F8" s="14" t="s">
+      <c r="F8" s="7" t="s">
         <v>80</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A9" s="3">
+        <v>5</v>
+      </c>
+      <c r="B9" s="4">
+        <v>45846</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10" s="3">
+        <v>6</v>
+      </c>
+      <c r="B10" s="4">
+        <v>45846</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>82</v>
       </c>
     </row>
   </sheetData>
@@ -1942,9 +2009,45 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DFE7F21C-61D1-4BE0-82A8-5BFBA9052C50}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="8.88671875" style="15"/>
+    <col min="2" max="2" width="15" style="16" customWidth="1"/>
+    <col min="3" max="3" width="43.33203125" style="17" customWidth="1"/>
+    <col min="4" max="4" width="53.6640625" style="17" customWidth="1"/>
+    <col min="5" max="16384" width="8.88671875" style="17"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" s="15" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="15" t="s">
+        <v>77</v>
+      </c>
+      <c r="B1" s="16" t="s">
+        <v>78</v>
+      </c>
+      <c r="C1" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1" s="15" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="115.2" x14ac:dyDescent="0.3">
+      <c r="A2" s="3">
+        <v>1</v>
+      </c>
+      <c r="B2" s="4">
+        <v>45846</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Updated the clean_data and data_io for easier file management. Created split_data module to split the dataset. Documentation of python files added in excel.
</commit_message>
<xml_diff>
--- a/documentation/under65_ai_project_documentations.xlsx
+++ b/documentation/under65_ai_project_documentations.xlsx
@@ -8,17 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jarpy\Documents\portfolio_projects\under65_stroke_risk_ai_tool\documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD8A912B-843A-43C2-BBBB-D00BB4A253C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4441D302-DF95-4CF5-8615-AE8B57A89B23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20610" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="2" xr2:uid="{B009FAC1-510D-4360-8356-4F13549178C2}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{B009FAC1-510D-4360-8356-4F13549178C2}"/>
   </bookViews>
   <sheets>
     <sheet name="Project Overview" sheetId="1" r:id="rId1"/>
     <sheet name="column_info" sheetId="6" r:id="rId2"/>
     <sheet name="cleaning_log" sheetId="2" r:id="rId3"/>
     <sheet name="eda_log" sheetId="3" r:id="rId4"/>
-    <sheet name="Sheet1" sheetId="5" r:id="rId5"/>
-    <sheet name="Sheet4" sheetId="4" r:id="rId6"/>
+    <sheet name="model_testing_template" sheetId="5" r:id="rId5"/>
+    <sheet name="python_log" sheetId="4" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="136">
   <si>
     <t>Under 65 AI Stroke Risk Assessment Tool</t>
   </si>
@@ -533,12 +533,116 @@
   <si>
     <t>No duplicates found (excluding id).</t>
   </si>
+  <si>
+    <t>Variations:
+1. Skewed continuous vs log transformed continuous
+2. SMOTE-TOMEK vs Non SMOTE</t>
+  </si>
+  <si>
+    <t>Filename</t>
+  </si>
+  <si>
+    <t>Definition</t>
+  </si>
+  <si>
+    <t>Return</t>
+  </si>
+  <si>
+    <t>data_io.py</t>
+  </si>
+  <si>
+    <t>Script for managing loading and saving of datasets</t>
+  </si>
+  <si>
+    <t>Definition Funciton</t>
+  </si>
+  <si>
+    <t>Load the raw data (original) csv</t>
+  </si>
+  <si>
+    <t>load_clean_data(filename="name of file")</t>
+  </si>
+  <si>
+    <t>load_raw_data(filepath="path to raw data")</t>
+  </si>
+  <si>
+    <t>dataframe</t>
+  </si>
+  <si>
+    <t>load the data requested using the file name, assumed cleaned</t>
+  </si>
+  <si>
+    <t>save_clean_data(df, filename="name of file")</t>
+  </si>
+  <si>
+    <t>Save the df into a csv using provided filename</t>
+  </si>
+  <si>
+    <t>data_cleaning.py</t>
+  </si>
+  <si>
+    <t>Preliminary Python-side cleaning process that standardize the text field and remove duplicates (assumed basic cleaning done by SQL)</t>
+  </si>
+  <si>
+    <t>inspect_data(df)</t>
+  </si>
+  <si>
+    <t>Uses info, describe, and isnull().sum() to show the column data types, number summary of continuous data, and null count for each column.</t>
+  </si>
+  <si>
+    <t>standardize_text_fields(df)</t>
+  </si>
+  <si>
+    <t>Standardize categorical columns to lowercase, trimmed, and replace in-between spaces with underscore.</t>
+  </si>
+  <si>
+    <t>remove_duplicates(df):</t>
+  </si>
+  <si>
+    <t>Removes any duplicate row while preserving the first instance (excluding id column)</t>
+  </si>
+  <si>
+    <t>clean_data()</t>
+  </si>
+  <si>
+    <t>Automate the process using the definitions of the module</t>
+  </si>
+  <si>
+    <t>split_data.py</t>
+  </si>
+  <si>
+    <t>Split the dataset into training and test sets</t>
+  </si>
+  <si>
+    <t>split_feature_target(df)</t>
+  </si>
+  <si>
+    <t>X,y</t>
+  </si>
+  <si>
+    <t>Splits the dataset into the feature columns (X) and the target columns (y)</t>
+  </si>
+  <si>
+    <t>train_test_stratified_split(X,y)</t>
+  </si>
+  <si>
+    <t>X_train, X_test, y_train, y_test</t>
+  </si>
+  <si>
+    <t>Split the dataset into 80/20 ratio (train/test), stratified to preserve ratio of no stroke / stroke</t>
+  </si>
+  <si>
+    <t>split_dataset()</t>
+  </si>
+  <si>
+    <t>Automates the split_data process and save the training and test set into individual csv files for consistency.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -585,6 +689,12 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Consolas"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="3">
@@ -637,7 +747,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -659,6 +769,15 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -682,13 +801,31 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1024,341 +1161,448 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{15FBF6C5-CE5C-424B-B4D7-C4EA3C1E0FE1}">
-  <dimension ref="A1:J27"/>
+  <dimension ref="A1:T27"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:10" ht="18" x14ac:dyDescent="0.35">
-      <c r="A1" s="8" t="s">
+    <row r="1" spans="1:20" ht="18" x14ac:dyDescent="0.35">
+      <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
-      <c r="H1" s="8"/>
-      <c r="I1" s="8"/>
-      <c r="J1" s="8"/>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A2" s="9" t="s">
+      <c r="B1" s="11"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
+      <c r="F1" s="11"/>
+      <c r="G1" s="11"/>
+      <c r="H1" s="11"/>
+      <c r="I1" s="11"/>
+      <c r="J1" s="11"/>
+    </row>
+    <row r="2" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A2" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="10"/>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="10"/>
-      <c r="F2" s="10"/>
-      <c r="G2" s="10"/>
-      <c r="H2" s="10"/>
-      <c r="I2" s="10"/>
-      <c r="J2" s="10"/>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A3" s="10"/>
-      <c r="B3" s="10"/>
-      <c r="C3" s="10"/>
-      <c r="D3" s="10"/>
-      <c r="E3" s="10"/>
-      <c r="F3" s="10"/>
-      <c r="G3" s="10"/>
-      <c r="H3" s="10"/>
-      <c r="I3" s="10"/>
-      <c r="J3" s="10"/>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A4" s="10"/>
-      <c r="B4" s="10"/>
-      <c r="C4" s="10"/>
-      <c r="D4" s="10"/>
-      <c r="E4" s="10"/>
-      <c r="F4" s="10"/>
-      <c r="G4" s="10"/>
-      <c r="H4" s="10"/>
-      <c r="I4" s="10"/>
-      <c r="J4" s="10"/>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A5" s="10"/>
-      <c r="B5" s="10"/>
-      <c r="C5" s="10"/>
-      <c r="D5" s="10"/>
-      <c r="E5" s="10"/>
-      <c r="F5" s="10"/>
-      <c r="G5" s="10"/>
-      <c r="H5" s="10"/>
-      <c r="I5" s="10"/>
-      <c r="J5" s="10"/>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A6" s="10"/>
-      <c r="B6" s="10"/>
-      <c r="C6" s="10"/>
-      <c r="D6" s="10"/>
-      <c r="E6" s="10"/>
-      <c r="F6" s="10"/>
-      <c r="G6" s="10"/>
-      <c r="H6" s="10"/>
-      <c r="I6" s="10"/>
-      <c r="J6" s="10"/>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A7" s="10"/>
-      <c r="B7" s="10"/>
-      <c r="C7" s="10"/>
-      <c r="D7" s="10"/>
-      <c r="E7" s="10"/>
-      <c r="F7" s="10"/>
-      <c r="G7" s="10"/>
-      <c r="H7" s="10"/>
-      <c r="I7" s="10"/>
-      <c r="J7" s="10"/>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A8" s="10"/>
-      <c r="B8" s="10"/>
-      <c r="C8" s="10"/>
-      <c r="D8" s="10"/>
-      <c r="E8" s="10"/>
-      <c r="F8" s="10"/>
-      <c r="G8" s="10"/>
-      <c r="H8" s="10"/>
-      <c r="I8" s="10"/>
-      <c r="J8" s="10"/>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A9" s="10"/>
-      <c r="B9" s="10"/>
-      <c r="C9" s="10"/>
-      <c r="D9" s="10"/>
-      <c r="E9" s="10"/>
-      <c r="F9" s="10"/>
-      <c r="G9" s="10"/>
-      <c r="H9" s="10"/>
-      <c r="I9" s="10"/>
-      <c r="J9" s="10"/>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A10" s="10"/>
-      <c r="B10" s="10"/>
-      <c r="C10" s="10"/>
-      <c r="D10" s="10"/>
-      <c r="E10" s="10"/>
-      <c r="F10" s="10"/>
-      <c r="G10" s="10"/>
-      <c r="H10" s="10"/>
-      <c r="I10" s="10"/>
-      <c r="J10" s="10"/>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A11" s="10"/>
-      <c r="B11" s="10"/>
-      <c r="C11" s="10"/>
-      <c r="D11" s="10"/>
-      <c r="E11" s="10"/>
-      <c r="F11" s="10"/>
-      <c r="G11" s="10"/>
-      <c r="H11" s="10"/>
-      <c r="I11" s="10"/>
-      <c r="J11" s="10"/>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="10"/>
-      <c r="B12" s="10"/>
-      <c r="C12" s="10"/>
-      <c r="D12" s="10"/>
-      <c r="E12" s="10"/>
-      <c r="F12" s="10"/>
-      <c r="G12" s="10"/>
-      <c r="H12" s="10"/>
-      <c r="I12" s="10"/>
-      <c r="J12" s="10"/>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A13" s="10"/>
-      <c r="B13" s="10"/>
-      <c r="C13" s="10"/>
-      <c r="D13" s="10"/>
-      <c r="E13" s="10"/>
-      <c r="F13" s="10"/>
-      <c r="G13" s="10"/>
-      <c r="H13" s="10"/>
-      <c r="I13" s="10"/>
-      <c r="J13" s="10"/>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A14" s="10"/>
-      <c r="B14" s="10"/>
-      <c r="C14" s="10"/>
-      <c r="D14" s="10"/>
-      <c r="E14" s="10"/>
-      <c r="F14" s="10"/>
-      <c r="G14" s="10"/>
-      <c r="H14" s="10"/>
-      <c r="I14" s="10"/>
-      <c r="J14" s="10"/>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A15" s="10"/>
-      <c r="B15" s="10"/>
-      <c r="C15" s="10"/>
-      <c r="D15" s="10"/>
-      <c r="E15" s="10"/>
-      <c r="F15" s="10"/>
-      <c r="G15" s="10"/>
-      <c r="H15" s="10"/>
-      <c r="I15" s="10"/>
-      <c r="J15" s="10"/>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="10"/>
-      <c r="B16" s="10"/>
-      <c r="C16" s="10"/>
-      <c r="D16" s="10"/>
-      <c r="E16" s="10"/>
-      <c r="F16" s="10"/>
-      <c r="G16" s="10"/>
-      <c r="H16" s="10"/>
-      <c r="I16" s="10"/>
-      <c r="J16" s="10"/>
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="13"/>
+      <c r="F2" s="13"/>
+      <c r="G2" s="13"/>
+      <c r="H2" s="13"/>
+      <c r="I2" s="13"/>
+      <c r="J2" s="13"/>
+      <c r="M2" s="19" t="s">
+        <v>102</v>
+      </c>
+      <c r="N2" s="18"/>
+      <c r="O2" s="18"/>
+      <c r="P2" s="18"/>
+      <c r="Q2" s="18"/>
+      <c r="R2" s="18"/>
+      <c r="S2" s="18"/>
+      <c r="T2" s="18"/>
+    </row>
+    <row r="3" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A3" s="13"/>
+      <c r="B3" s="13"/>
+      <c r="C3" s="13"/>
+      <c r="D3" s="13"/>
+      <c r="E3" s="13"/>
+      <c r="F3" s="13"/>
+      <c r="G3" s="13"/>
+      <c r="H3" s="13"/>
+      <c r="I3" s="13"/>
+      <c r="J3" s="13"/>
+      <c r="M3" s="18"/>
+      <c r="N3" s="18"/>
+      <c r="O3" s="18"/>
+      <c r="P3" s="18"/>
+      <c r="Q3" s="18"/>
+      <c r="R3" s="18"/>
+      <c r="S3" s="18"/>
+      <c r="T3" s="18"/>
+    </row>
+    <row r="4" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A4" s="13"/>
+      <c r="B4" s="13"/>
+      <c r="C4" s="13"/>
+      <c r="D4" s="13"/>
+      <c r="E4" s="13"/>
+      <c r="F4" s="13"/>
+      <c r="G4" s="13"/>
+      <c r="H4" s="13"/>
+      <c r="I4" s="13"/>
+      <c r="J4" s="13"/>
+      <c r="M4" s="18"/>
+      <c r="N4" s="18"/>
+      <c r="O4" s="18"/>
+      <c r="P4" s="18"/>
+      <c r="Q4" s="18"/>
+      <c r="R4" s="18"/>
+      <c r="S4" s="18"/>
+      <c r="T4" s="18"/>
+    </row>
+    <row r="5" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A5" s="13"/>
+      <c r="B5" s="13"/>
+      <c r="C5" s="13"/>
+      <c r="D5" s="13"/>
+      <c r="E5" s="13"/>
+      <c r="F5" s="13"/>
+      <c r="G5" s="13"/>
+      <c r="H5" s="13"/>
+      <c r="I5" s="13"/>
+      <c r="J5" s="13"/>
+      <c r="M5" s="18"/>
+      <c r="N5" s="18"/>
+      <c r="O5" s="18"/>
+      <c r="P5" s="18"/>
+      <c r="Q5" s="18"/>
+      <c r="R5" s="18"/>
+      <c r="S5" s="18"/>
+      <c r="T5" s="18"/>
+    </row>
+    <row r="6" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A6" s="13"/>
+      <c r="B6" s="13"/>
+      <c r="C6" s="13"/>
+      <c r="D6" s="13"/>
+      <c r="E6" s="13"/>
+      <c r="F6" s="13"/>
+      <c r="G6" s="13"/>
+      <c r="H6" s="13"/>
+      <c r="I6" s="13"/>
+      <c r="J6" s="13"/>
+      <c r="M6" s="18"/>
+      <c r="N6" s="18"/>
+      <c r="O6" s="18"/>
+      <c r="P6" s="18"/>
+      <c r="Q6" s="18"/>
+      <c r="R6" s="18"/>
+      <c r="S6" s="18"/>
+      <c r="T6" s="18"/>
+    </row>
+    <row r="7" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A7" s="13"/>
+      <c r="B7" s="13"/>
+      <c r="C7" s="13"/>
+      <c r="D7" s="13"/>
+      <c r="E7" s="13"/>
+      <c r="F7" s="13"/>
+      <c r="G7" s="13"/>
+      <c r="H7" s="13"/>
+      <c r="I7" s="13"/>
+      <c r="J7" s="13"/>
+      <c r="M7" s="18"/>
+      <c r="N7" s="18"/>
+      <c r="O7" s="18"/>
+      <c r="P7" s="18"/>
+      <c r="Q7" s="18"/>
+      <c r="R7" s="18"/>
+      <c r="S7" s="18"/>
+      <c r="T7" s="18"/>
+    </row>
+    <row r="8" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A8" s="13"/>
+      <c r="B8" s="13"/>
+      <c r="C8" s="13"/>
+      <c r="D8" s="13"/>
+      <c r="E8" s="13"/>
+      <c r="F8" s="13"/>
+      <c r="G8" s="13"/>
+      <c r="H8" s="13"/>
+      <c r="I8" s="13"/>
+      <c r="J8" s="13"/>
+      <c r="M8" s="18"/>
+      <c r="N8" s="18"/>
+      <c r="O8" s="18"/>
+      <c r="P8" s="18"/>
+      <c r="Q8" s="18"/>
+      <c r="R8" s="18"/>
+      <c r="S8" s="18"/>
+      <c r="T8" s="18"/>
+    </row>
+    <row r="9" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A9" s="13"/>
+      <c r="B9" s="13"/>
+      <c r="C9" s="13"/>
+      <c r="D9" s="13"/>
+      <c r="E9" s="13"/>
+      <c r="F9" s="13"/>
+      <c r="G9" s="13"/>
+      <c r="H9" s="13"/>
+      <c r="I9" s="13"/>
+      <c r="J9" s="13"/>
+      <c r="M9" s="18"/>
+      <c r="N9" s="18"/>
+      <c r="O9" s="18"/>
+      <c r="P9" s="18"/>
+      <c r="Q9" s="18"/>
+      <c r="R9" s="18"/>
+      <c r="S9" s="18"/>
+      <c r="T9" s="18"/>
+    </row>
+    <row r="10" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A10" s="13"/>
+      <c r="B10" s="13"/>
+      <c r="C10" s="13"/>
+      <c r="D10" s="13"/>
+      <c r="E10" s="13"/>
+      <c r="F10" s="13"/>
+      <c r="G10" s="13"/>
+      <c r="H10" s="13"/>
+      <c r="I10" s="13"/>
+      <c r="J10" s="13"/>
+      <c r="M10" s="18"/>
+      <c r="N10" s="18"/>
+      <c r="O10" s="18"/>
+      <c r="P10" s="18"/>
+      <c r="Q10" s="18"/>
+      <c r="R10" s="18"/>
+      <c r="S10" s="18"/>
+      <c r="T10" s="18"/>
+    </row>
+    <row r="11" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A11" s="13"/>
+      <c r="B11" s="13"/>
+      <c r="C11" s="13"/>
+      <c r="D11" s="13"/>
+      <c r="E11" s="13"/>
+      <c r="F11" s="13"/>
+      <c r="G11" s="13"/>
+      <c r="H11" s="13"/>
+      <c r="I11" s="13"/>
+      <c r="J11" s="13"/>
+      <c r="M11" s="18"/>
+      <c r="N11" s="18"/>
+      <c r="O11" s="18"/>
+      <c r="P11" s="18"/>
+      <c r="Q11" s="18"/>
+      <c r="R11" s="18"/>
+      <c r="S11" s="18"/>
+      <c r="T11" s="18"/>
+    </row>
+    <row r="12" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A12" s="13"/>
+      <c r="B12" s="13"/>
+      <c r="C12" s="13"/>
+      <c r="D12" s="13"/>
+      <c r="E12" s="13"/>
+      <c r="F12" s="13"/>
+      <c r="G12" s="13"/>
+      <c r="H12" s="13"/>
+      <c r="I12" s="13"/>
+      <c r="J12" s="13"/>
+      <c r="M12" s="18"/>
+      <c r="N12" s="18"/>
+      <c r="O12" s="18"/>
+      <c r="P12" s="18"/>
+      <c r="Q12" s="18"/>
+      <c r="R12" s="18"/>
+      <c r="S12" s="18"/>
+      <c r="T12" s="18"/>
+    </row>
+    <row r="13" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A13" s="13"/>
+      <c r="B13" s="13"/>
+      <c r="C13" s="13"/>
+      <c r="D13" s="13"/>
+      <c r="E13" s="13"/>
+      <c r="F13" s="13"/>
+      <c r="G13" s="13"/>
+      <c r="H13" s="13"/>
+      <c r="I13" s="13"/>
+      <c r="J13" s="13"/>
+      <c r="M13" s="18"/>
+      <c r="N13" s="18"/>
+      <c r="O13" s="18"/>
+      <c r="P13" s="18"/>
+      <c r="Q13" s="18"/>
+      <c r="R13" s="18"/>
+      <c r="S13" s="18"/>
+      <c r="T13" s="18"/>
+    </row>
+    <row r="14" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A14" s="13"/>
+      <c r="B14" s="13"/>
+      <c r="C14" s="13"/>
+      <c r="D14" s="13"/>
+      <c r="E14" s="13"/>
+      <c r="F14" s="13"/>
+      <c r="G14" s="13"/>
+      <c r="H14" s="13"/>
+      <c r="I14" s="13"/>
+      <c r="J14" s="13"/>
+      <c r="M14" s="18"/>
+      <c r="N14" s="18"/>
+      <c r="O14" s="18"/>
+      <c r="P14" s="18"/>
+      <c r="Q14" s="18"/>
+      <c r="R14" s="18"/>
+      <c r="S14" s="18"/>
+      <c r="T14" s="18"/>
+    </row>
+    <row r="15" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A15" s="13"/>
+      <c r="B15" s="13"/>
+      <c r="C15" s="13"/>
+      <c r="D15" s="13"/>
+      <c r="E15" s="13"/>
+      <c r="F15" s="13"/>
+      <c r="G15" s="13"/>
+      <c r="H15" s="13"/>
+      <c r="I15" s="13"/>
+      <c r="J15" s="13"/>
+    </row>
+    <row r="16" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A16" s="13"/>
+      <c r="B16" s="13"/>
+      <c r="C16" s="13"/>
+      <c r="D16" s="13"/>
+      <c r="E16" s="13"/>
+      <c r="F16" s="13"/>
+      <c r="G16" s="13"/>
+      <c r="H16" s="13"/>
+      <c r="I16" s="13"/>
+      <c r="J16" s="13"/>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A17" s="10"/>
-      <c r="B17" s="10"/>
-      <c r="C17" s="10"/>
-      <c r="D17" s="10"/>
-      <c r="E17" s="10"/>
-      <c r="F17" s="10"/>
-      <c r="G17" s="10"/>
-      <c r="H17" s="10"/>
-      <c r="I17" s="10"/>
-      <c r="J17" s="10"/>
+      <c r="A17" s="13"/>
+      <c r="B17" s="13"/>
+      <c r="C17" s="13"/>
+      <c r="D17" s="13"/>
+      <c r="E17" s="13"/>
+      <c r="F17" s="13"/>
+      <c r="G17" s="13"/>
+      <c r="H17" s="13"/>
+      <c r="I17" s="13"/>
+      <c r="J17" s="13"/>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A18" s="10"/>
-      <c r="B18" s="10"/>
-      <c r="C18" s="10"/>
-      <c r="D18" s="10"/>
-      <c r="E18" s="10"/>
-      <c r="F18" s="10"/>
-      <c r="G18" s="10"/>
-      <c r="H18" s="10"/>
-      <c r="I18" s="10"/>
-      <c r="J18" s="10"/>
+      <c r="A18" s="13"/>
+      <c r="B18" s="13"/>
+      <c r="C18" s="13"/>
+      <c r="D18" s="13"/>
+      <c r="E18" s="13"/>
+      <c r="F18" s="13"/>
+      <c r="G18" s="13"/>
+      <c r="H18" s="13"/>
+      <c r="I18" s="13"/>
+      <c r="J18" s="13"/>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A19" s="10"/>
-      <c r="B19" s="10"/>
-      <c r="C19" s="10"/>
-      <c r="D19" s="10"/>
-      <c r="E19" s="10"/>
-      <c r="F19" s="10"/>
-      <c r="G19" s="10"/>
-      <c r="H19" s="10"/>
-      <c r="I19" s="10"/>
-      <c r="J19" s="10"/>
+      <c r="A19" s="13"/>
+      <c r="B19" s="13"/>
+      <c r="C19" s="13"/>
+      <c r="D19" s="13"/>
+      <c r="E19" s="13"/>
+      <c r="F19" s="13"/>
+      <c r="G19" s="13"/>
+      <c r="H19" s="13"/>
+      <c r="I19" s="13"/>
+      <c r="J19" s="13"/>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A20" s="10"/>
-      <c r="B20" s="10"/>
-      <c r="C20" s="10"/>
-      <c r="D20" s="10"/>
-      <c r="E20" s="10"/>
-      <c r="F20" s="10"/>
-      <c r="G20" s="10"/>
-      <c r="H20" s="10"/>
-      <c r="I20" s="10"/>
-      <c r="J20" s="10"/>
+      <c r="A20" s="13"/>
+      <c r="B20" s="13"/>
+      <c r="C20" s="13"/>
+      <c r="D20" s="13"/>
+      <c r="E20" s="13"/>
+      <c r="F20" s="13"/>
+      <c r="G20" s="13"/>
+      <c r="H20" s="13"/>
+      <c r="I20" s="13"/>
+      <c r="J20" s="13"/>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A21" s="10"/>
-      <c r="B21" s="10"/>
-      <c r="C21" s="10"/>
-      <c r="D21" s="10"/>
-      <c r="E21" s="10"/>
-      <c r="F21" s="10"/>
-      <c r="G21" s="10"/>
-      <c r="H21" s="10"/>
-      <c r="I21" s="10"/>
-      <c r="J21" s="10"/>
+      <c r="A21" s="13"/>
+      <c r="B21" s="13"/>
+      <c r="C21" s="13"/>
+      <c r="D21" s="13"/>
+      <c r="E21" s="13"/>
+      <c r="F21" s="13"/>
+      <c r="G21" s="13"/>
+      <c r="H21" s="13"/>
+      <c r="I21" s="13"/>
+      <c r="J21" s="13"/>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A22" s="10"/>
-      <c r="B22" s="10"/>
-      <c r="C22" s="10"/>
-      <c r="D22" s="10"/>
-      <c r="E22" s="10"/>
-      <c r="F22" s="10"/>
-      <c r="G22" s="10"/>
-      <c r="H22" s="10"/>
-      <c r="I22" s="10"/>
-      <c r="J22" s="10"/>
+      <c r="A22" s="13"/>
+      <c r="B22" s="13"/>
+      <c r="C22" s="13"/>
+      <c r="D22" s="13"/>
+      <c r="E22" s="13"/>
+      <c r="F22" s="13"/>
+      <c r="G22" s="13"/>
+      <c r="H22" s="13"/>
+      <c r="I22" s="13"/>
+      <c r="J22" s="13"/>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A23" s="10"/>
-      <c r="B23" s="10"/>
-      <c r="C23" s="10"/>
-      <c r="D23" s="10"/>
-      <c r="E23" s="10"/>
-      <c r="F23" s="10"/>
-      <c r="G23" s="10"/>
-      <c r="H23" s="10"/>
-      <c r="I23" s="10"/>
-      <c r="J23" s="10"/>
+      <c r="A23" s="13"/>
+      <c r="B23" s="13"/>
+      <c r="C23" s="13"/>
+      <c r="D23" s="13"/>
+      <c r="E23" s="13"/>
+      <c r="F23" s="13"/>
+      <c r="G23" s="13"/>
+      <c r="H23" s="13"/>
+      <c r="I23" s="13"/>
+      <c r="J23" s="13"/>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A24" s="10"/>
-      <c r="B24" s="10"/>
-      <c r="C24" s="10"/>
-      <c r="D24" s="10"/>
-      <c r="E24" s="10"/>
-      <c r="F24" s="10"/>
-      <c r="G24" s="10"/>
-      <c r="H24" s="10"/>
-      <c r="I24" s="10"/>
-      <c r="J24" s="10"/>
+      <c r="A24" s="13"/>
+      <c r="B24" s="13"/>
+      <c r="C24" s="13"/>
+      <c r="D24" s="13"/>
+      <c r="E24" s="13"/>
+      <c r="F24" s="13"/>
+      <c r="G24" s="13"/>
+      <c r="H24" s="13"/>
+      <c r="I24" s="13"/>
+      <c r="J24" s="13"/>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A25" s="10"/>
-      <c r="B25" s="10"/>
-      <c r="C25" s="10"/>
-      <c r="D25" s="10"/>
-      <c r="E25" s="10"/>
-      <c r="F25" s="10"/>
-      <c r="G25" s="10"/>
-      <c r="H25" s="10"/>
-      <c r="I25" s="10"/>
-      <c r="J25" s="10"/>
+      <c r="A25" s="13"/>
+      <c r="B25" s="13"/>
+      <c r="C25" s="13"/>
+      <c r="D25" s="13"/>
+      <c r="E25" s="13"/>
+      <c r="F25" s="13"/>
+      <c r="G25" s="13"/>
+      <c r="H25" s="13"/>
+      <c r="I25" s="13"/>
+      <c r="J25" s="13"/>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A26" s="10"/>
-      <c r="B26" s="10"/>
-      <c r="C26" s="10"/>
-      <c r="D26" s="10"/>
-      <c r="E26" s="10"/>
-      <c r="F26" s="10"/>
-      <c r="G26" s="10"/>
-      <c r="H26" s="10"/>
-      <c r="I26" s="10"/>
-      <c r="J26" s="10"/>
+      <c r="A26" s="13"/>
+      <c r="B26" s="13"/>
+      <c r="C26" s="13"/>
+      <c r="D26" s="13"/>
+      <c r="E26" s="13"/>
+      <c r="F26" s="13"/>
+      <c r="G26" s="13"/>
+      <c r="H26" s="13"/>
+      <c r="I26" s="13"/>
+      <c r="J26" s="13"/>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A27" s="10"/>
-      <c r="B27" s="10"/>
-      <c r="C27" s="10"/>
-      <c r="D27" s="10"/>
-      <c r="E27" s="10"/>
-      <c r="F27" s="10"/>
-      <c r="G27" s="10"/>
-      <c r="H27" s="10"/>
-      <c r="I27" s="10"/>
-      <c r="J27" s="10"/>
+      <c r="A27" s="13"/>
+      <c r="B27" s="13"/>
+      <c r="C27" s="13"/>
+      <c r="D27" s="13"/>
+      <c r="E27" s="13"/>
+      <c r="F27" s="13"/>
+      <c r="G27" s="13"/>
+      <c r="H27" s="13"/>
+      <c r="I27" s="13"/>
+      <c r="J27" s="13"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A2:J27"/>
+    <mergeCell ref="M2:T14"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1380,14 +1624,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:7" ht="21" x14ac:dyDescent="0.3">
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
-      <c r="G1" s="11"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
     </row>
     <row r="2" spans="2:7" s="3" customFormat="1" ht="18" x14ac:dyDescent="0.3">
       <c r="B2" s="5" t="s">
@@ -1648,14 +1892,14 @@
       </c>
     </row>
     <row r="15" spans="2:7" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="12" t="s">
+      <c r="B15" s="15" t="s">
         <v>56</v>
       </c>
-      <c r="C15" s="12"/>
-      <c r="D15" s="12"/>
-      <c r="E15" s="12"/>
-      <c r="F15" s="12"/>
-      <c r="G15" s="12"/>
+      <c r="C15" s="15"/>
+      <c r="D15" s="15"/>
+      <c r="E15" s="15"/>
+      <c r="F15" s="15"/>
+      <c r="G15" s="15"/>
     </row>
     <row r="16" spans="2:7" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="5" t="s">
@@ -1828,14 +2072,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="16" t="s">
         <v>89</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
     </row>
     <row r="2" spans="1:6" s="3" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A2" s="7" t="s">
@@ -1935,14 +2179,14 @@
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" s="14" t="s">
+      <c r="A7" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="B7" s="14"/>
-      <c r="C7" s="14"/>
-      <c r="D7" s="14"/>
-      <c r="E7" s="14"/>
-      <c r="F7" s="14"/>
+      <c r="B7" s="17"/>
+      <c r="C7" s="17"/>
+      <c r="D7" s="17"/>
+      <c r="E7" s="17"/>
+      <c r="F7" s="17"/>
     </row>
     <row r="8" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A8" s="7" t="s">
@@ -2012,24 +2256,24 @@
   <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.88671875" style="15"/>
-    <col min="2" max="2" width="15" style="16" customWidth="1"/>
-    <col min="3" max="3" width="43.33203125" style="17" customWidth="1"/>
-    <col min="4" max="4" width="53.6640625" style="17" customWidth="1"/>
-    <col min="5" max="16384" width="8.88671875" style="17"/>
+    <col min="1" max="1" width="8.88671875" style="8"/>
+    <col min="2" max="2" width="15" style="9" customWidth="1"/>
+    <col min="3" max="3" width="43.33203125" style="10" customWidth="1"/>
+    <col min="4" max="4" width="53.6640625" style="10" customWidth="1"/>
+    <col min="5" max="16384" width="8.88671875" style="10"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="15" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="15" t="s">
+    <row r="1" spans="1:4" s="8" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="8" t="s">
         <v>77</v>
       </c>
-      <c r="B1" s="16" t="s">
+      <c r="B1" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="C1" s="15" t="s">
+      <c r="C1" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="D1" s="15" t="s">
+      <c r="D1" s="8" t="s">
         <v>95</v>
       </c>
     </row>
@@ -2066,9 +2310,230 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC828414-FBE3-46EC-BDC7-F550F4CA42BA}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="8.88671875" style="1"/>
+    <col min="2" max="2" width="17.88671875" style="20" customWidth="1"/>
+    <col min="3" max="3" width="26.6640625" style="1" customWidth="1"/>
+    <col min="4" max="5" width="35.6640625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="26.5546875" style="1" customWidth="1"/>
+    <col min="7" max="7" width="53.44140625" style="1" customWidth="1"/>
+    <col min="8" max="16384" width="8.88671875" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" s="3" customFormat="1" ht="18" x14ac:dyDescent="0.3">
+      <c r="A1" s="21" t="s">
+        <v>77</v>
+      </c>
+      <c r="B1" s="22" t="s">
+        <v>78</v>
+      </c>
+      <c r="C1" s="21" t="s">
+        <v>103</v>
+      </c>
+      <c r="D1" s="21" t="s">
+        <v>5</v>
+      </c>
+      <c r="E1" s="21" t="s">
+        <v>104</v>
+      </c>
+      <c r="F1" s="21" t="s">
+        <v>105</v>
+      </c>
+      <c r="G1" s="21" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="23">
+        <v>1</v>
+      </c>
+      <c r="B2" s="24">
+        <v>45846</v>
+      </c>
+      <c r="C2" s="23" t="s">
+        <v>106</v>
+      </c>
+      <c r="D2" s="25" t="s">
+        <v>107</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3" s="23"/>
+      <c r="B3" s="24"/>
+      <c r="C3" s="23"/>
+      <c r="D3" s="25"/>
+      <c r="E3" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A4" s="23"/>
+      <c r="B4" s="24"/>
+      <c r="C4" s="23"/>
+      <c r="D4" s="25"/>
+      <c r="E4" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="23">
+        <v>2</v>
+      </c>
+      <c r="B5" s="24">
+        <v>45846</v>
+      </c>
+      <c r="C5" s="23" t="s">
+        <v>116</v>
+      </c>
+      <c r="D5" s="25" t="s">
+        <v>117</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A6" s="23"/>
+      <c r="B6" s="24"/>
+      <c r="C6" s="23"/>
+      <c r="D6" s="25"/>
+      <c r="E6" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A7" s="23"/>
+      <c r="B7" s="24"/>
+      <c r="C7" s="23"/>
+      <c r="D7" s="25"/>
+      <c r="E7" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A8" s="23"/>
+      <c r="B8" s="24"/>
+      <c r="C8" s="23"/>
+      <c r="D8" s="25"/>
+      <c r="E8" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A9" s="23">
+        <v>3</v>
+      </c>
+      <c r="B9" s="24">
+        <v>45846</v>
+      </c>
+      <c r="C9" s="23" t="s">
+        <v>126</v>
+      </c>
+      <c r="D9" s="25" t="s">
+        <v>127</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="28.8" x14ac:dyDescent="0.25">
+      <c r="A10" s="23"/>
+      <c r="B10" s="24"/>
+      <c r="C10" s="23"/>
+      <c r="D10" s="25"/>
+      <c r="E10" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="F10" s="26" t="s">
+        <v>132</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A11" s="23"/>
+      <c r="B11" s="24"/>
+      <c r="C11" s="23"/>
+      <c r="D11" s="25"/>
+      <c r="E11" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>135</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="12">
+    <mergeCell ref="A9:A11"/>
+    <mergeCell ref="B9:B11"/>
+    <mergeCell ref="C9:C11"/>
+    <mergeCell ref="D9:D11"/>
+    <mergeCell ref="A2:A4"/>
+    <mergeCell ref="B2:B4"/>
+    <mergeCell ref="C2:C4"/>
+    <mergeCell ref="D2:D4"/>
+    <mergeCell ref="A5:A8"/>
+    <mergeCell ref="B5:B8"/>
+    <mergeCell ref="C5:C8"/>
+    <mergeCell ref="D5:D8"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Finished preprocess_data.py complete with smote, normalize, and impute. Updated documentation. Updated data_io for series vs df.
</commit_message>
<xml_diff>
--- a/documentation/under65_ai_project_documentations.xlsx
+++ b/documentation/under65_ai_project_documentations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jarpy\Documents\portfolio_projects\under65_stroke_risk_ai_tool\documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4441D302-DF95-4CF5-8615-AE8B57A89B23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70C455F6-8350-4096-AC3A-1AF9C6C5BCFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{B009FAC1-510D-4360-8356-4F13549178C2}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="172">
   <si>
     <t>Under 65 AI Stroke Risk Assessment Tool</t>
   </si>
@@ -637,6 +637,129 @@
   <si>
     <t>Automates the split_data process and save the training and test set into individual csv files for consistency.</t>
   </si>
+  <si>
+    <t>Dropped gender and residence_type columns</t>
+  </si>
+  <si>
+    <t>Based on previous data analysis work on the under 65 dataset, Chi-Square Test showed that gender and residence_type are statistically insignificant features when it comes to predicting stroke.</t>
+  </si>
+  <si>
+    <t>Categorical Encoding</t>
+  </si>
+  <si>
+    <t>One-Hot ecoded all categorical features using the trianing data as reference. Drop_first=True used to avoid multicollinearity.</t>
+  </si>
+  <si>
+    <t>Imputation (two methods)</t>
+  </si>
+  <si>
+    <t>Class balancing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SMOTE-Tomek applied to training set only (if user indicated yes). </t>
+  </si>
+  <si>
+    <t>Normalization</t>
+  </si>
+  <si>
+    <t xml:space="preserve">StandardScaler used on age, bmi, and avg_glucose_level. Fit on training set only to avoid leakage. </t>
+  </si>
+  <si>
+    <t>1. Median value bmi imputation is used by default and  second method is Random Forest regressor. 
+2. Model saved as rf_bmi_imputer.joblib
+3. Transform data stored as float64 for downstream compatibility.</t>
+  </si>
+  <si>
+    <t>Final Sanity Check</t>
+  </si>
+  <si>
+    <t>1. All features confirmed as float64. 
+2. Nulls = 0 
+3. Training/testing sets aligned. 
+4. Column order and scaler saved.</t>
+  </si>
+  <si>
+    <t>preprocess_data</t>
+  </si>
+  <si>
+    <t>Prepare the data for modeling:
+1. Retireve the split data
+2. Drop insignificant features
+3. One-hot Encode categoricals
+4. Impute missing values (median/rf)
+5. Smote (if requested)
+6. Verify preprocessed data</t>
+  </si>
+  <si>
+    <t>drop)insignificant_features(X_train, X_test)</t>
+  </si>
+  <si>
+    <t>X_train, X_test</t>
+  </si>
+  <si>
+    <t>Drops the identified insignificant features from statistical analysis.</t>
+  </si>
+  <si>
+    <t>encode_categorical_features(X_train, X_test)</t>
+  </si>
+  <si>
+    <t>X_train_encoded, X_test_encoded</t>
+  </si>
+  <si>
+    <t>apply_smote(X_train, y_train)</t>
+  </si>
+  <si>
+    <t>X_train_resampled, y_train_resampled</t>
+  </si>
+  <si>
+    <t>If the user chose to use smote, this definition applies SMOTE-Tomek to resample the training sets.</t>
+  </si>
+  <si>
+    <t>normalize_continuous(X_train_impute, X_test_impute)</t>
+  </si>
+  <si>
+    <t>X_train_impute, X_test_impute</t>
+  </si>
+  <si>
+    <t>1. One-hot Encode categorical features and trurn them as float64 type for downstream compatibility.
+2. Saved the column order for later use.</t>
+  </si>
+  <si>
+    <t>1. Normalizes the previously imputed feature sets (X) using StandardScaler.
+2. Scaler is saved for future use.</t>
+  </si>
+  <si>
+    <t>random_forest_impute_bmi(X_train, X_test)</t>
+  </si>
+  <si>
+    <t>1. Uses a Random Forest regressor to impute the missing bmi values.
+2. Saves the rf_impute model for future use.</t>
+  </si>
+  <si>
+    <t>median_impute(X_train, X_test)</t>
+  </si>
+  <si>
+    <t>1. Imputes the missing bmi with the median value.
+2. Saves the imputer for future use.</t>
+  </si>
+  <si>
+    <t>check_shapes_and_nulls(X_train, X_test, y_train, y_test)</t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>Checks and prints the shape, description, and number of null values of the datasets for verification.</t>
+  </si>
+  <si>
+    <t>preprocess_data(smote=False, rf_impute=False)</t>
+  </si>
+  <si>
+    <t>X_train_resampled, X_test_impute, y_train_resampled, y_test</t>
+  </si>
+  <si>
+    <t>Automates all preprocessing stages based on user preference (smote, rf_impute).</t>
+  </si>
 </sst>
 </file>
 
@@ -711,7 +834,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -743,11 +866,20 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -779,6 +911,18 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -788,6 +932,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -800,21 +950,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -824,8 +959,20 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1165,438 +1312,438 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:20" ht="18" x14ac:dyDescent="0.35">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
-      <c r="G1" s="11"/>
-      <c r="H1" s="11"/>
-      <c r="I1" s="11"/>
-      <c r="J1" s="11"/>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
+      <c r="H1" s="15"/>
+      <c r="I1" s="15"/>
+      <c r="J1" s="15"/>
     </row>
     <row r="2" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="13"/>
-      <c r="C2" s="13"/>
-      <c r="D2" s="13"/>
-      <c r="E2" s="13"/>
-      <c r="F2" s="13"/>
-      <c r="G2" s="13"/>
-      <c r="H2" s="13"/>
-      <c r="I2" s="13"/>
-      <c r="J2" s="13"/>
-      <c r="M2" s="19" t="s">
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="17"/>
+      <c r="F2" s="17"/>
+      <c r="G2" s="17"/>
+      <c r="H2" s="17"/>
+      <c r="I2" s="17"/>
+      <c r="J2" s="17"/>
+      <c r="M2" s="18" t="s">
         <v>102</v>
       </c>
-      <c r="N2" s="18"/>
-      <c r="O2" s="18"/>
-      <c r="P2" s="18"/>
-      <c r="Q2" s="18"/>
-      <c r="R2" s="18"/>
-      <c r="S2" s="18"/>
-      <c r="T2" s="18"/>
+      <c r="N2" s="19"/>
+      <c r="O2" s="19"/>
+      <c r="P2" s="19"/>
+      <c r="Q2" s="19"/>
+      <c r="R2" s="19"/>
+      <c r="S2" s="19"/>
+      <c r="T2" s="19"/>
     </row>
     <row r="3" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A3" s="13"/>
-      <c r="B3" s="13"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
-      <c r="E3" s="13"/>
-      <c r="F3" s="13"/>
-      <c r="G3" s="13"/>
-      <c r="H3" s="13"/>
-      <c r="I3" s="13"/>
-      <c r="J3" s="13"/>
-      <c r="M3" s="18"/>
-      <c r="N3" s="18"/>
-      <c r="O3" s="18"/>
-      <c r="P3" s="18"/>
-      <c r="Q3" s="18"/>
-      <c r="R3" s="18"/>
-      <c r="S3" s="18"/>
-      <c r="T3" s="18"/>
+      <c r="A3" s="17"/>
+      <c r="B3" s="17"/>
+      <c r="C3" s="17"/>
+      <c r="D3" s="17"/>
+      <c r="E3" s="17"/>
+      <c r="F3" s="17"/>
+      <c r="G3" s="17"/>
+      <c r="H3" s="17"/>
+      <c r="I3" s="17"/>
+      <c r="J3" s="17"/>
+      <c r="M3" s="19"/>
+      <c r="N3" s="19"/>
+      <c r="O3" s="19"/>
+      <c r="P3" s="19"/>
+      <c r="Q3" s="19"/>
+      <c r="R3" s="19"/>
+      <c r="S3" s="19"/>
+      <c r="T3" s="19"/>
     </row>
     <row r="4" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A4" s="13"/>
-      <c r="B4" s="13"/>
-      <c r="C4" s="13"/>
-      <c r="D4" s="13"/>
-      <c r="E4" s="13"/>
-      <c r="F4" s="13"/>
-      <c r="G4" s="13"/>
-      <c r="H4" s="13"/>
-      <c r="I4" s="13"/>
-      <c r="J4" s="13"/>
-      <c r="M4" s="18"/>
-      <c r="N4" s="18"/>
-      <c r="O4" s="18"/>
-      <c r="P4" s="18"/>
-      <c r="Q4" s="18"/>
-      <c r="R4" s="18"/>
-      <c r="S4" s="18"/>
-      <c r="T4" s="18"/>
+      <c r="A4" s="17"/>
+      <c r="B4" s="17"/>
+      <c r="C4" s="17"/>
+      <c r="D4" s="17"/>
+      <c r="E4" s="17"/>
+      <c r="F4" s="17"/>
+      <c r="G4" s="17"/>
+      <c r="H4" s="17"/>
+      <c r="I4" s="17"/>
+      <c r="J4" s="17"/>
+      <c r="M4" s="19"/>
+      <c r="N4" s="19"/>
+      <c r="O4" s="19"/>
+      <c r="P4" s="19"/>
+      <c r="Q4" s="19"/>
+      <c r="R4" s="19"/>
+      <c r="S4" s="19"/>
+      <c r="T4" s="19"/>
     </row>
     <row r="5" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A5" s="13"/>
-      <c r="B5" s="13"/>
-      <c r="C5" s="13"/>
-      <c r="D5" s="13"/>
-      <c r="E5" s="13"/>
-      <c r="F5" s="13"/>
-      <c r="G5" s="13"/>
-      <c r="H5" s="13"/>
-      <c r="I5" s="13"/>
-      <c r="J5" s="13"/>
-      <c r="M5" s="18"/>
-      <c r="N5" s="18"/>
-      <c r="O5" s="18"/>
-      <c r="P5" s="18"/>
-      <c r="Q5" s="18"/>
-      <c r="R5" s="18"/>
-      <c r="S5" s="18"/>
-      <c r="T5" s="18"/>
+      <c r="A5" s="17"/>
+      <c r="B5" s="17"/>
+      <c r="C5" s="17"/>
+      <c r="D5" s="17"/>
+      <c r="E5" s="17"/>
+      <c r="F5" s="17"/>
+      <c r="G5" s="17"/>
+      <c r="H5" s="17"/>
+      <c r="I5" s="17"/>
+      <c r="J5" s="17"/>
+      <c r="M5" s="19"/>
+      <c r="N5" s="19"/>
+      <c r="O5" s="19"/>
+      <c r="P5" s="19"/>
+      <c r="Q5" s="19"/>
+      <c r="R5" s="19"/>
+      <c r="S5" s="19"/>
+      <c r="T5" s="19"/>
     </row>
     <row r="6" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A6" s="13"/>
-      <c r="B6" s="13"/>
-      <c r="C6" s="13"/>
-      <c r="D6" s="13"/>
-      <c r="E6" s="13"/>
-      <c r="F6" s="13"/>
-      <c r="G6" s="13"/>
-      <c r="H6" s="13"/>
-      <c r="I6" s="13"/>
-      <c r="J6" s="13"/>
-      <c r="M6" s="18"/>
-      <c r="N6" s="18"/>
-      <c r="O6" s="18"/>
-      <c r="P6" s="18"/>
-      <c r="Q6" s="18"/>
-      <c r="R6" s="18"/>
-      <c r="S6" s="18"/>
-      <c r="T6" s="18"/>
+      <c r="A6" s="17"/>
+      <c r="B6" s="17"/>
+      <c r="C6" s="17"/>
+      <c r="D6" s="17"/>
+      <c r="E6" s="17"/>
+      <c r="F6" s="17"/>
+      <c r="G6" s="17"/>
+      <c r="H6" s="17"/>
+      <c r="I6" s="17"/>
+      <c r="J6" s="17"/>
+      <c r="M6" s="19"/>
+      <c r="N6" s="19"/>
+      <c r="O6" s="19"/>
+      <c r="P6" s="19"/>
+      <c r="Q6" s="19"/>
+      <c r="R6" s="19"/>
+      <c r="S6" s="19"/>
+      <c r="T6" s="19"/>
     </row>
     <row r="7" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A7" s="13"/>
-      <c r="B7" s="13"/>
-      <c r="C7" s="13"/>
-      <c r="D7" s="13"/>
-      <c r="E7" s="13"/>
-      <c r="F7" s="13"/>
-      <c r="G7" s="13"/>
-      <c r="H7" s="13"/>
-      <c r="I7" s="13"/>
-      <c r="J7" s="13"/>
-      <c r="M7" s="18"/>
-      <c r="N7" s="18"/>
-      <c r="O7" s="18"/>
-      <c r="P7" s="18"/>
-      <c r="Q7" s="18"/>
-      <c r="R7" s="18"/>
-      <c r="S7" s="18"/>
-      <c r="T7" s="18"/>
+      <c r="A7" s="17"/>
+      <c r="B7" s="17"/>
+      <c r="C7" s="17"/>
+      <c r="D7" s="17"/>
+      <c r="E7" s="17"/>
+      <c r="F7" s="17"/>
+      <c r="G7" s="17"/>
+      <c r="H7" s="17"/>
+      <c r="I7" s="17"/>
+      <c r="J7" s="17"/>
+      <c r="M7" s="19"/>
+      <c r="N7" s="19"/>
+      <c r="O7" s="19"/>
+      <c r="P7" s="19"/>
+      <c r="Q7" s="19"/>
+      <c r="R7" s="19"/>
+      <c r="S7" s="19"/>
+      <c r="T7" s="19"/>
     </row>
     <row r="8" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A8" s="13"/>
-      <c r="B8" s="13"/>
-      <c r="C8" s="13"/>
-      <c r="D8" s="13"/>
-      <c r="E8" s="13"/>
-      <c r="F8" s="13"/>
-      <c r="G8" s="13"/>
-      <c r="H8" s="13"/>
-      <c r="I8" s="13"/>
-      <c r="J8" s="13"/>
-      <c r="M8" s="18"/>
-      <c r="N8" s="18"/>
-      <c r="O8" s="18"/>
-      <c r="P8" s="18"/>
-      <c r="Q8" s="18"/>
-      <c r="R8" s="18"/>
-      <c r="S8" s="18"/>
-      <c r="T8" s="18"/>
+      <c r="A8" s="17"/>
+      <c r="B8" s="17"/>
+      <c r="C8" s="17"/>
+      <c r="D8" s="17"/>
+      <c r="E8" s="17"/>
+      <c r="F8" s="17"/>
+      <c r="G8" s="17"/>
+      <c r="H8" s="17"/>
+      <c r="I8" s="17"/>
+      <c r="J8" s="17"/>
+      <c r="M8" s="19"/>
+      <c r="N8" s="19"/>
+      <c r="O8" s="19"/>
+      <c r="P8" s="19"/>
+      <c r="Q8" s="19"/>
+      <c r="R8" s="19"/>
+      <c r="S8" s="19"/>
+      <c r="T8" s="19"/>
     </row>
     <row r="9" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A9" s="13"/>
-      <c r="B9" s="13"/>
-      <c r="C9" s="13"/>
-      <c r="D9" s="13"/>
-      <c r="E9" s="13"/>
-      <c r="F9" s="13"/>
-      <c r="G9" s="13"/>
-      <c r="H9" s="13"/>
-      <c r="I9" s="13"/>
-      <c r="J9" s="13"/>
-      <c r="M9" s="18"/>
-      <c r="N9" s="18"/>
-      <c r="O9" s="18"/>
-      <c r="P9" s="18"/>
-      <c r="Q9" s="18"/>
-      <c r="R9" s="18"/>
-      <c r="S9" s="18"/>
-      <c r="T9" s="18"/>
+      <c r="A9" s="17"/>
+      <c r="B9" s="17"/>
+      <c r="C9" s="17"/>
+      <c r="D9" s="17"/>
+      <c r="E9" s="17"/>
+      <c r="F9" s="17"/>
+      <c r="G9" s="17"/>
+      <c r="H9" s="17"/>
+      <c r="I9" s="17"/>
+      <c r="J9" s="17"/>
+      <c r="M9" s="19"/>
+      <c r="N9" s="19"/>
+      <c r="O9" s="19"/>
+      <c r="P9" s="19"/>
+      <c r="Q9" s="19"/>
+      <c r="R9" s="19"/>
+      <c r="S9" s="19"/>
+      <c r="T9" s="19"/>
     </row>
     <row r="10" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A10" s="13"/>
-      <c r="B10" s="13"/>
-      <c r="C10" s="13"/>
-      <c r="D10" s="13"/>
-      <c r="E10" s="13"/>
-      <c r="F10" s="13"/>
-      <c r="G10" s="13"/>
-      <c r="H10" s="13"/>
-      <c r="I10" s="13"/>
-      <c r="J10" s="13"/>
-      <c r="M10" s="18"/>
-      <c r="N10" s="18"/>
-      <c r="O10" s="18"/>
-      <c r="P10" s="18"/>
-      <c r="Q10" s="18"/>
-      <c r="R10" s="18"/>
-      <c r="S10" s="18"/>
-      <c r="T10" s="18"/>
+      <c r="A10" s="17"/>
+      <c r="B10" s="17"/>
+      <c r="C10" s="17"/>
+      <c r="D10" s="17"/>
+      <c r="E10" s="17"/>
+      <c r="F10" s="17"/>
+      <c r="G10" s="17"/>
+      <c r="H10" s="17"/>
+      <c r="I10" s="17"/>
+      <c r="J10" s="17"/>
+      <c r="M10" s="19"/>
+      <c r="N10" s="19"/>
+      <c r="O10" s="19"/>
+      <c r="P10" s="19"/>
+      <c r="Q10" s="19"/>
+      <c r="R10" s="19"/>
+      <c r="S10" s="19"/>
+      <c r="T10" s="19"/>
     </row>
     <row r="11" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A11" s="13"/>
-      <c r="B11" s="13"/>
-      <c r="C11" s="13"/>
-      <c r="D11" s="13"/>
-      <c r="E11" s="13"/>
-      <c r="F11" s="13"/>
-      <c r="G11" s="13"/>
-      <c r="H11" s="13"/>
-      <c r="I11" s="13"/>
-      <c r="J11" s="13"/>
-      <c r="M11" s="18"/>
-      <c r="N11" s="18"/>
-      <c r="O11" s="18"/>
-      <c r="P11" s="18"/>
-      <c r="Q11" s="18"/>
-      <c r="R11" s="18"/>
-      <c r="S11" s="18"/>
-      <c r="T11" s="18"/>
+      <c r="A11" s="17"/>
+      <c r="B11" s="17"/>
+      <c r="C11" s="17"/>
+      <c r="D11" s="17"/>
+      <c r="E11" s="17"/>
+      <c r="F11" s="17"/>
+      <c r="G11" s="17"/>
+      <c r="H11" s="17"/>
+      <c r="I11" s="17"/>
+      <c r="J11" s="17"/>
+      <c r="M11" s="19"/>
+      <c r="N11" s="19"/>
+      <c r="O11" s="19"/>
+      <c r="P11" s="19"/>
+      <c r="Q11" s="19"/>
+      <c r="R11" s="19"/>
+      <c r="S11" s="19"/>
+      <c r="T11" s="19"/>
     </row>
     <row r="12" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A12" s="13"/>
-      <c r="B12" s="13"/>
-      <c r="C12" s="13"/>
-      <c r="D12" s="13"/>
-      <c r="E12" s="13"/>
-      <c r="F12" s="13"/>
-      <c r="G12" s="13"/>
-      <c r="H12" s="13"/>
-      <c r="I12" s="13"/>
-      <c r="J12" s="13"/>
-      <c r="M12" s="18"/>
-      <c r="N12" s="18"/>
-      <c r="O12" s="18"/>
-      <c r="P12" s="18"/>
-      <c r="Q12" s="18"/>
-      <c r="R12" s="18"/>
-      <c r="S12" s="18"/>
-      <c r="T12" s="18"/>
+      <c r="A12" s="17"/>
+      <c r="B12" s="17"/>
+      <c r="C12" s="17"/>
+      <c r="D12" s="17"/>
+      <c r="E12" s="17"/>
+      <c r="F12" s="17"/>
+      <c r="G12" s="17"/>
+      <c r="H12" s="17"/>
+      <c r="I12" s="17"/>
+      <c r="J12" s="17"/>
+      <c r="M12" s="19"/>
+      <c r="N12" s="19"/>
+      <c r="O12" s="19"/>
+      <c r="P12" s="19"/>
+      <c r="Q12" s="19"/>
+      <c r="R12" s="19"/>
+      <c r="S12" s="19"/>
+      <c r="T12" s="19"/>
     </row>
     <row r="13" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A13" s="13"/>
-      <c r="B13" s="13"/>
-      <c r="C13" s="13"/>
-      <c r="D13" s="13"/>
-      <c r="E13" s="13"/>
-      <c r="F13" s="13"/>
-      <c r="G13" s="13"/>
-      <c r="H13" s="13"/>
-      <c r="I13" s="13"/>
-      <c r="J13" s="13"/>
-      <c r="M13" s="18"/>
-      <c r="N13" s="18"/>
-      <c r="O13" s="18"/>
-      <c r="P13" s="18"/>
-      <c r="Q13" s="18"/>
-      <c r="R13" s="18"/>
-      <c r="S13" s="18"/>
-      <c r="T13" s="18"/>
+      <c r="A13" s="17"/>
+      <c r="B13" s="17"/>
+      <c r="C13" s="17"/>
+      <c r="D13" s="17"/>
+      <c r="E13" s="17"/>
+      <c r="F13" s="17"/>
+      <c r="G13" s="17"/>
+      <c r="H13" s="17"/>
+      <c r="I13" s="17"/>
+      <c r="J13" s="17"/>
+      <c r="M13" s="19"/>
+      <c r="N13" s="19"/>
+      <c r="O13" s="19"/>
+      <c r="P13" s="19"/>
+      <c r="Q13" s="19"/>
+      <c r="R13" s="19"/>
+      <c r="S13" s="19"/>
+      <c r="T13" s="19"/>
     </row>
     <row r="14" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A14" s="13"/>
-      <c r="B14" s="13"/>
-      <c r="C14" s="13"/>
-      <c r="D14" s="13"/>
-      <c r="E14" s="13"/>
-      <c r="F14" s="13"/>
-      <c r="G14" s="13"/>
-      <c r="H14" s="13"/>
-      <c r="I14" s="13"/>
-      <c r="J14" s="13"/>
-      <c r="M14" s="18"/>
-      <c r="N14" s="18"/>
-      <c r="O14" s="18"/>
-      <c r="P14" s="18"/>
-      <c r="Q14" s="18"/>
-      <c r="R14" s="18"/>
-      <c r="S14" s="18"/>
-      <c r="T14" s="18"/>
+      <c r="A14" s="17"/>
+      <c r="B14" s="17"/>
+      <c r="C14" s="17"/>
+      <c r="D14" s="17"/>
+      <c r="E14" s="17"/>
+      <c r="F14" s="17"/>
+      <c r="G14" s="17"/>
+      <c r="H14" s="17"/>
+      <c r="I14" s="17"/>
+      <c r="J14" s="17"/>
+      <c r="M14" s="19"/>
+      <c r="N14" s="19"/>
+      <c r="O14" s="19"/>
+      <c r="P14" s="19"/>
+      <c r="Q14" s="19"/>
+      <c r="R14" s="19"/>
+      <c r="S14" s="19"/>
+      <c r="T14" s="19"/>
     </row>
     <row r="15" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A15" s="13"/>
-      <c r="B15" s="13"/>
-      <c r="C15" s="13"/>
-      <c r="D15" s="13"/>
-      <c r="E15" s="13"/>
-      <c r="F15" s="13"/>
-      <c r="G15" s="13"/>
-      <c r="H15" s="13"/>
-      <c r="I15" s="13"/>
-      <c r="J15" s="13"/>
+      <c r="A15" s="17"/>
+      <c r="B15" s="17"/>
+      <c r="C15" s="17"/>
+      <c r="D15" s="17"/>
+      <c r="E15" s="17"/>
+      <c r="F15" s="17"/>
+      <c r="G15" s="17"/>
+      <c r="H15" s="17"/>
+      <c r="I15" s="17"/>
+      <c r="J15" s="17"/>
     </row>
     <row r="16" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A16" s="13"/>
-      <c r="B16" s="13"/>
-      <c r="C16" s="13"/>
-      <c r="D16" s="13"/>
-      <c r="E16" s="13"/>
-      <c r="F16" s="13"/>
-      <c r="G16" s="13"/>
-      <c r="H16" s="13"/>
-      <c r="I16" s="13"/>
-      <c r="J16" s="13"/>
+      <c r="A16" s="17"/>
+      <c r="B16" s="17"/>
+      <c r="C16" s="17"/>
+      <c r="D16" s="17"/>
+      <c r="E16" s="17"/>
+      <c r="F16" s="17"/>
+      <c r="G16" s="17"/>
+      <c r="H16" s="17"/>
+      <c r="I16" s="17"/>
+      <c r="J16" s="17"/>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A17" s="13"/>
-      <c r="B17" s="13"/>
-      <c r="C17" s="13"/>
-      <c r="D17" s="13"/>
-      <c r="E17" s="13"/>
-      <c r="F17" s="13"/>
-      <c r="G17" s="13"/>
-      <c r="H17" s="13"/>
-      <c r="I17" s="13"/>
-      <c r="J17" s="13"/>
+      <c r="A17" s="17"/>
+      <c r="B17" s="17"/>
+      <c r="C17" s="17"/>
+      <c r="D17" s="17"/>
+      <c r="E17" s="17"/>
+      <c r="F17" s="17"/>
+      <c r="G17" s="17"/>
+      <c r="H17" s="17"/>
+      <c r="I17" s="17"/>
+      <c r="J17" s="17"/>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A18" s="13"/>
-      <c r="B18" s="13"/>
-      <c r="C18" s="13"/>
-      <c r="D18" s="13"/>
-      <c r="E18" s="13"/>
-      <c r="F18" s="13"/>
-      <c r="G18" s="13"/>
-      <c r="H18" s="13"/>
-      <c r="I18" s="13"/>
-      <c r="J18" s="13"/>
+      <c r="A18" s="17"/>
+      <c r="B18" s="17"/>
+      <c r="C18" s="17"/>
+      <c r="D18" s="17"/>
+      <c r="E18" s="17"/>
+      <c r="F18" s="17"/>
+      <c r="G18" s="17"/>
+      <c r="H18" s="17"/>
+      <c r="I18" s="17"/>
+      <c r="J18" s="17"/>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A19" s="13"/>
-      <c r="B19" s="13"/>
-      <c r="C19" s="13"/>
-      <c r="D19" s="13"/>
-      <c r="E19" s="13"/>
-      <c r="F19" s="13"/>
-      <c r="G19" s="13"/>
-      <c r="H19" s="13"/>
-      <c r="I19" s="13"/>
-      <c r="J19" s="13"/>
+      <c r="A19" s="17"/>
+      <c r="B19" s="17"/>
+      <c r="C19" s="17"/>
+      <c r="D19" s="17"/>
+      <c r="E19" s="17"/>
+      <c r="F19" s="17"/>
+      <c r="G19" s="17"/>
+      <c r="H19" s="17"/>
+      <c r="I19" s="17"/>
+      <c r="J19" s="17"/>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A20" s="13"/>
-      <c r="B20" s="13"/>
-      <c r="C20" s="13"/>
-      <c r="D20" s="13"/>
-      <c r="E20" s="13"/>
-      <c r="F20" s="13"/>
-      <c r="G20" s="13"/>
-      <c r="H20" s="13"/>
-      <c r="I20" s="13"/>
-      <c r="J20" s="13"/>
+      <c r="A20" s="17"/>
+      <c r="B20" s="17"/>
+      <c r="C20" s="17"/>
+      <c r="D20" s="17"/>
+      <c r="E20" s="17"/>
+      <c r="F20" s="17"/>
+      <c r="G20" s="17"/>
+      <c r="H20" s="17"/>
+      <c r="I20" s="17"/>
+      <c r="J20" s="17"/>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A21" s="13"/>
-      <c r="B21" s="13"/>
-      <c r="C21" s="13"/>
-      <c r="D21" s="13"/>
-      <c r="E21" s="13"/>
-      <c r="F21" s="13"/>
-      <c r="G21" s="13"/>
-      <c r="H21" s="13"/>
-      <c r="I21" s="13"/>
-      <c r="J21" s="13"/>
+      <c r="A21" s="17"/>
+      <c r="B21" s="17"/>
+      <c r="C21" s="17"/>
+      <c r="D21" s="17"/>
+      <c r="E21" s="17"/>
+      <c r="F21" s="17"/>
+      <c r="G21" s="17"/>
+      <c r="H21" s="17"/>
+      <c r="I21" s="17"/>
+      <c r="J21" s="17"/>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A22" s="13"/>
-      <c r="B22" s="13"/>
-      <c r="C22" s="13"/>
-      <c r="D22" s="13"/>
-      <c r="E22" s="13"/>
-      <c r="F22" s="13"/>
-      <c r="G22" s="13"/>
-      <c r="H22" s="13"/>
-      <c r="I22" s="13"/>
-      <c r="J22" s="13"/>
+      <c r="A22" s="17"/>
+      <c r="B22" s="17"/>
+      <c r="C22" s="17"/>
+      <c r="D22" s="17"/>
+      <c r="E22" s="17"/>
+      <c r="F22" s="17"/>
+      <c r="G22" s="17"/>
+      <c r="H22" s="17"/>
+      <c r="I22" s="17"/>
+      <c r="J22" s="17"/>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A23" s="13"/>
-      <c r="B23" s="13"/>
-      <c r="C23" s="13"/>
-      <c r="D23" s="13"/>
-      <c r="E23" s="13"/>
-      <c r="F23" s="13"/>
-      <c r="G23" s="13"/>
-      <c r="H23" s="13"/>
-      <c r="I23" s="13"/>
-      <c r="J23" s="13"/>
+      <c r="A23" s="17"/>
+      <c r="B23" s="17"/>
+      <c r="C23" s="17"/>
+      <c r="D23" s="17"/>
+      <c r="E23" s="17"/>
+      <c r="F23" s="17"/>
+      <c r="G23" s="17"/>
+      <c r="H23" s="17"/>
+      <c r="I23" s="17"/>
+      <c r="J23" s="17"/>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A24" s="13"/>
-      <c r="B24" s="13"/>
-      <c r="C24" s="13"/>
-      <c r="D24" s="13"/>
-      <c r="E24" s="13"/>
-      <c r="F24" s="13"/>
-      <c r="G24" s="13"/>
-      <c r="H24" s="13"/>
-      <c r="I24" s="13"/>
-      <c r="J24" s="13"/>
+      <c r="A24" s="17"/>
+      <c r="B24" s="17"/>
+      <c r="C24" s="17"/>
+      <c r="D24" s="17"/>
+      <c r="E24" s="17"/>
+      <c r="F24" s="17"/>
+      <c r="G24" s="17"/>
+      <c r="H24" s="17"/>
+      <c r="I24" s="17"/>
+      <c r="J24" s="17"/>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A25" s="13"/>
-      <c r="B25" s="13"/>
-      <c r="C25" s="13"/>
-      <c r="D25" s="13"/>
-      <c r="E25" s="13"/>
-      <c r="F25" s="13"/>
-      <c r="G25" s="13"/>
-      <c r="H25" s="13"/>
-      <c r="I25" s="13"/>
-      <c r="J25" s="13"/>
+      <c r="A25" s="17"/>
+      <c r="B25" s="17"/>
+      <c r="C25" s="17"/>
+      <c r="D25" s="17"/>
+      <c r="E25" s="17"/>
+      <c r="F25" s="17"/>
+      <c r="G25" s="17"/>
+      <c r="H25" s="17"/>
+      <c r="I25" s="17"/>
+      <c r="J25" s="17"/>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A26" s="13"/>
-      <c r="B26" s="13"/>
-      <c r="C26" s="13"/>
-      <c r="D26" s="13"/>
-      <c r="E26" s="13"/>
-      <c r="F26" s="13"/>
-      <c r="G26" s="13"/>
-      <c r="H26" s="13"/>
-      <c r="I26" s="13"/>
-      <c r="J26" s="13"/>
+      <c r="A26" s="17"/>
+      <c r="B26" s="17"/>
+      <c r="C26" s="17"/>
+      <c r="D26" s="17"/>
+      <c r="E26" s="17"/>
+      <c r="F26" s="17"/>
+      <c r="G26" s="17"/>
+      <c r="H26" s="17"/>
+      <c r="I26" s="17"/>
+      <c r="J26" s="17"/>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A27" s="13"/>
-      <c r="B27" s="13"/>
-      <c r="C27" s="13"/>
-      <c r="D27" s="13"/>
-      <c r="E27" s="13"/>
-      <c r="F27" s="13"/>
-      <c r="G27" s="13"/>
-      <c r="H27" s="13"/>
-      <c r="I27" s="13"/>
-      <c r="J27" s="13"/>
+      <c r="A27" s="17"/>
+      <c r="B27" s="17"/>
+      <c r="C27" s="17"/>
+      <c r="D27" s="17"/>
+      <c r="E27" s="17"/>
+      <c r="F27" s="17"/>
+      <c r="G27" s="17"/>
+      <c r="H27" s="17"/>
+      <c r="I27" s="17"/>
+      <c r="J27" s="17"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -1624,14 +1771,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:7" ht="21" x14ac:dyDescent="0.3">
-      <c r="B1" s="14" t="s">
+      <c r="B1" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
-      <c r="G1" s="14"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
     </row>
     <row r="2" spans="2:7" s="3" customFormat="1" ht="18" x14ac:dyDescent="0.3">
       <c r="B2" s="5" t="s">
@@ -1892,14 +2039,14 @@
       </c>
     </row>
     <row r="15" spans="2:7" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="15" t="s">
+      <c r="B15" s="21" t="s">
         <v>56</v>
       </c>
-      <c r="C15" s="15"/>
-      <c r="D15" s="15"/>
-      <c r="E15" s="15"/>
-      <c r="F15" s="15"/>
-      <c r="G15" s="15"/>
+      <c r="C15" s="21"/>
+      <c r="D15" s="21"/>
+      <c r="E15" s="21"/>
+      <c r="F15" s="21"/>
+      <c r="G15" s="21"/>
     </row>
     <row r="16" spans="2:7" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="5" t="s">
@@ -2072,14 +2219,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="22" t="s">
         <v>89</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
     </row>
     <row r="2" spans="1:6" s="3" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A2" s="7" t="s">
@@ -2179,14 +2326,14 @@
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" s="17" t="s">
+      <c r="A7" s="23" t="s">
         <v>94</v>
       </c>
-      <c r="B7" s="17"/>
-      <c r="C7" s="17"/>
-      <c r="D7" s="17"/>
-      <c r="E7" s="17"/>
-      <c r="F7" s="17"/>
+      <c r="B7" s="23"/>
+      <c r="C7" s="23"/>
+      <c r="D7" s="23"/>
+      <c r="E7" s="23"/>
+      <c r="F7" s="23"/>
     </row>
     <row r="8" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A8" s="7" t="s">
@@ -2253,7 +2400,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DFE7F21C-61D1-4BE0-82A8-5BFBA9052C50}">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.88671875" style="8"/>
@@ -2289,6 +2436,90 @@
       </c>
       <c r="D2" s="1" t="s">
         <v>97</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A3" s="8">
+        <v>2</v>
+      </c>
+      <c r="B3" s="9">
+        <v>45846</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>136</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A4" s="8">
+        <v>3</v>
+      </c>
+      <c r="B4" s="9">
+        <v>45847</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>138</v>
+      </c>
+      <c r="D4" s="10" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A5" s="8">
+        <v>4</v>
+      </c>
+      <c r="B5" s="9">
+        <v>45847</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>140</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" s="8">
+        <v>5</v>
+      </c>
+      <c r="B6" s="9">
+        <v>45847</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>141</v>
+      </c>
+      <c r="D6" s="10" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A7" s="8">
+        <v>6</v>
+      </c>
+      <c r="B7" s="9">
+        <v>45847</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>143</v>
+      </c>
+      <c r="D7" s="10" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A8" s="8">
+        <v>7</v>
+      </c>
+      <c r="B8" s="9">
+        <v>45847</v>
+      </c>
+      <c r="C8" s="10" t="s">
+        <v>146</v>
+      </c>
+      <c r="D8" s="10" t="s">
+        <v>147</v>
       </c>
     </row>
   </sheetData>
@@ -2310,52 +2541,53 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC828414-FBE3-46EC-BDC7-F550F4CA42BA}">
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.88671875" style="1"/>
-    <col min="2" max="2" width="17.88671875" style="20" customWidth="1"/>
+    <col min="2" max="2" width="17.88671875" style="11" customWidth="1"/>
     <col min="3" max="3" width="26.6640625" style="1" customWidth="1"/>
-    <col min="4" max="5" width="35.6640625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="35.6640625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="37.109375" style="1" customWidth="1"/>
     <col min="6" max="6" width="26.5546875" style="1" customWidth="1"/>
     <col min="7" max="7" width="53.44140625" style="1" customWidth="1"/>
     <col min="8" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" s="3" customFormat="1" ht="18" x14ac:dyDescent="0.3">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="12" t="s">
         <v>77</v>
       </c>
-      <c r="B1" s="22" t="s">
+      <c r="B1" s="13" t="s">
         <v>78</v>
       </c>
-      <c r="C1" s="21" t="s">
+      <c r="C1" s="12" t="s">
         <v>103</v>
       </c>
-      <c r="D1" s="21" t="s">
+      <c r="D1" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="E1" s="21" t="s">
+      <c r="E1" s="12" t="s">
         <v>104</v>
       </c>
-      <c r="F1" s="21" t="s">
+      <c r="F1" s="12" t="s">
         <v>105</v>
       </c>
-      <c r="G1" s="21" t="s">
+      <c r="G1" s="12" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="23">
+      <c r="A2" s="24">
         <v>1</v>
       </c>
-      <c r="B2" s="24">
+      <c r="B2" s="25">
         <v>45846</v>
       </c>
-      <c r="C2" s="23" t="s">
+      <c r="C2" s="24" t="s">
         <v>106</v>
       </c>
-      <c r="D2" s="25" t="s">
+      <c r="D2" s="26" t="s">
         <v>107</v>
       </c>
       <c r="E2" s="2" t="s">
@@ -2369,10 +2601,10 @@
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" s="23"/>
-      <c r="B3" s="24"/>
-      <c r="C3" s="23"/>
-      <c r="D3" s="25"/>
+      <c r="A3" s="24"/>
+      <c r="B3" s="25"/>
+      <c r="C3" s="24"/>
+      <c r="D3" s="26"/>
       <c r="E3" s="2" t="s">
         <v>110</v>
       </c>
@@ -2384,10 +2616,10 @@
       </c>
     </row>
     <row r="4" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A4" s="23"/>
-      <c r="B4" s="24"/>
-      <c r="C4" s="23"/>
-      <c r="D4" s="25"/>
+      <c r="A4" s="24"/>
+      <c r="B4" s="25"/>
+      <c r="C4" s="24"/>
+      <c r="D4" s="26"/>
       <c r="E4" s="2" t="s">
         <v>114</v>
       </c>
@@ -2399,16 +2631,16 @@
       </c>
     </row>
     <row r="5" spans="1:7" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="23">
+      <c r="A5" s="24">
         <v>2</v>
       </c>
-      <c r="B5" s="24">
+      <c r="B5" s="25">
         <v>45846</v>
       </c>
-      <c r="C5" s="23" t="s">
+      <c r="C5" s="24" t="s">
         <v>116</v>
       </c>
-      <c r="D5" s="25" t="s">
+      <c r="D5" s="26" t="s">
         <v>117</v>
       </c>
       <c r="E5" s="2" t="s">
@@ -2422,10 +2654,10 @@
       </c>
     </row>
     <row r="6" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A6" s="23"/>
-      <c r="B6" s="24"/>
-      <c r="C6" s="23"/>
-      <c r="D6" s="25"/>
+      <c r="A6" s="24"/>
+      <c r="B6" s="25"/>
+      <c r="C6" s="24"/>
+      <c r="D6" s="26"/>
       <c r="E6" s="2" t="s">
         <v>120</v>
       </c>
@@ -2437,10 +2669,10 @@
       </c>
     </row>
     <row r="7" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A7" s="23"/>
-      <c r="B7" s="24"/>
-      <c r="C7" s="23"/>
-      <c r="D7" s="25"/>
+      <c r="A7" s="24"/>
+      <c r="B7" s="25"/>
+      <c r="C7" s="24"/>
+      <c r="D7" s="26"/>
       <c r="E7" s="2" t="s">
         <v>122</v>
       </c>
@@ -2452,10 +2684,10 @@
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A8" s="23"/>
-      <c r="B8" s="24"/>
-      <c r="C8" s="23"/>
-      <c r="D8" s="25"/>
+      <c r="A8" s="24"/>
+      <c r="B8" s="25"/>
+      <c r="C8" s="24"/>
+      <c r="D8" s="26"/>
       <c r="E8" s="2" t="s">
         <v>124</v>
       </c>
@@ -2467,16 +2699,16 @@
       </c>
     </row>
     <row r="9" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A9" s="23">
+      <c r="A9" s="24">
         <v>3</v>
       </c>
-      <c r="B9" s="24">
+      <c r="B9" s="25">
         <v>45846</v>
       </c>
-      <c r="C9" s="23" t="s">
+      <c r="C9" s="24" t="s">
         <v>126</v>
       </c>
-      <c r="D9" s="25" t="s">
+      <c r="D9" s="26" t="s">
         <v>127</v>
       </c>
       <c r="E9" s="2" t="s">
@@ -2490,14 +2722,14 @@
       </c>
     </row>
     <row r="10" spans="1:7" ht="28.8" x14ac:dyDescent="0.25">
-      <c r="A10" s="23"/>
-      <c r="B10" s="24"/>
-      <c r="C10" s="23"/>
-      <c r="D10" s="25"/>
+      <c r="A10" s="24"/>
+      <c r="B10" s="25"/>
+      <c r="C10" s="24"/>
+      <c r="D10" s="26"/>
       <c r="E10" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="F10" s="26" t="s">
+      <c r="F10" s="14" t="s">
         <v>132</v>
       </c>
       <c r="G10" s="2" t="s">
@@ -2505,10 +2737,10 @@
       </c>
     </row>
     <row r="11" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A11" s="23"/>
-      <c r="B11" s="24"/>
-      <c r="C11" s="23"/>
-      <c r="D11" s="25"/>
+      <c r="A11" s="24"/>
+      <c r="B11" s="25"/>
+      <c r="C11" s="24"/>
+      <c r="D11" s="26"/>
       <c r="E11" s="2" t="s">
         <v>134</v>
       </c>
@@ -2519,8 +2751,140 @@
         <v>135</v>
       </c>
     </row>
+    <row r="12" spans="1:7" ht="100.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="27">
+        <v>4</v>
+      </c>
+      <c r="B12" s="29">
+        <v>45846</v>
+      </c>
+      <c r="C12" s="27" t="s">
+        <v>148</v>
+      </c>
+      <c r="D12" s="31" t="s">
+        <v>149</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A13" s="23"/>
+      <c r="B13" s="28"/>
+      <c r="C13" s="23"/>
+      <c r="D13" s="30"/>
+      <c r="E13" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A14" s="23"/>
+      <c r="B14" s="28"/>
+      <c r="C14" s="23"/>
+      <c r="D14" s="30"/>
+      <c r="E14" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A15" s="23"/>
+      <c r="B15" s="28"/>
+      <c r="C15" s="23"/>
+      <c r="D15" s="30"/>
+      <c r="E15" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="G15" s="1" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A16" s="23"/>
+      <c r="B16" s="28"/>
+      <c r="C16" s="23"/>
+      <c r="D16" s="30"/>
+      <c r="E16" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="G16" s="1" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A17" s="23"/>
+      <c r="B17" s="28"/>
+      <c r="C17" s="23"/>
+      <c r="D17" s="30"/>
+      <c r="E17" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="G17" s="1" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A18" s="23"/>
+      <c r="B18" s="28"/>
+      <c r="C18" s="23"/>
+      <c r="D18" s="30"/>
+      <c r="E18" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="G18" s="1" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A19" s="23"/>
+      <c r="B19" s="28"/>
+      <c r="C19" s="23"/>
+      <c r="D19" s="30"/>
+      <c r="E19" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="G19" s="1" t="s">
+        <v>171</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="16">
+    <mergeCell ref="A12:A19"/>
+    <mergeCell ref="B12:B19"/>
+    <mergeCell ref="C12:C19"/>
+    <mergeCell ref="D12:D19"/>
     <mergeCell ref="A9:A11"/>
     <mergeCell ref="B9:B11"/>
     <mergeCell ref="C9:C11"/>

</xml_diff>